<commit_message>
feat: update template and download
</commit_message>
<xml_diff>
--- a/public/assets/templates/maintenance/battery.xlsx
+++ b/public/assets/templates/maintenance/battery.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\maintenance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCF15692-60E0-4E3C-B5DC-E9E8C71BD4B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D52223E1-D4CD-4365-B2A4-E41BA21E642A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{632ED090-5FEF-4C64-87E3-52D42BEDE752}"/>
   </bookViews>
@@ -451,7 +451,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -500,27 +500,84 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -528,12 +585,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -542,68 +593,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -986,54 +983,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="15" thickTop="1">
-      <c r="A1" s="40"/>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="43" t="s">
+      <c r="A1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="44"/>
-      <c r="R1" s="44"/>
-      <c r="S1" s="44"/>
-      <c r="T1" s="44"/>
-      <c r="U1" s="45"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
+      <c r="S1" s="29"/>
+      <c r="T1" s="29"/>
+      <c r="U1" s="30"/>
     </row>
     <row r="2" spans="1:21">
-      <c r="A2" s="42"/>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="46" t="s">
+      <c r="A2" s="26"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
-      <c r="L2" s="47"/>
-      <c r="M2" s="47"/>
-      <c r="N2" s="47"/>
-      <c r="O2" s="47"/>
-      <c r="P2" s="47"/>
-      <c r="Q2" s="47"/>
-      <c r="R2" s="47"/>
-      <c r="S2" s="47"/>
-      <c r="T2" s="47"/>
-      <c r="U2" s="48"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="32"/>
+      <c r="Q2" s="32"/>
+      <c r="R2" s="32"/>
+      <c r="S2" s="32"/>
+      <c r="T2" s="32"/>
+      <c r="U2" s="33"/>
     </row>
     <row r="3" spans="1:21">
       <c r="A3" s="1"/>
@@ -1041,14 +1038,14 @@
       <c r="U3" s="3"/>
     </row>
     <row r="4" spans="1:21">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="34"/>
       <c r="G4" s="4"/>
       <c r="H4" t="s">
         <v>3</v>
@@ -1076,14 +1073,14 @@
       <c r="U5" s="3"/>
     </row>
     <row r="6" spans="1:21">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="49"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="49"/>
-      <c r="F6" s="49"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
       <c r="G6" s="7"/>
       <c r="H6" t="s">
         <v>6</v>
@@ -1111,11 +1108,11 @@
       <c r="U8" s="3"/>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="38" t="s">
+      <c r="A9" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="39"/>
-      <c r="C9" s="39"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
       <c r="D9" s="9" t="s">
         <v>8</v>
       </c>
@@ -1172,159 +1169,159 @@
       </c>
     </row>
     <row r="10" spans="1:21">
-      <c r="A10" s="34" t="s">
+      <c r="A10" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="35"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="36"/>
-      <c r="G10" s="36"/>
-      <c r="H10" s="36"/>
-      <c r="I10" s="36"/>
-      <c r="J10" s="36"/>
-      <c r="K10" s="36"/>
-      <c r="L10" s="36"/>
-      <c r="M10" s="36"/>
-      <c r="N10" s="36"/>
-      <c r="O10" s="36"/>
-      <c r="P10" s="36"/>
-      <c r="Q10" s="36"/>
-      <c r="R10" s="36"/>
-      <c r="S10" s="36"/>
-      <c r="T10" s="36"/>
-      <c r="U10" s="37"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="23"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
+      <c r="M10" s="23"/>
+      <c r="N10" s="23"/>
+      <c r="O10" s="23"/>
+      <c r="P10" s="23"/>
+      <c r="Q10" s="23"/>
+      <c r="R10" s="23"/>
+      <c r="S10" s="23"/>
+      <c r="T10" s="23"/>
+      <c r="U10" s="35"/>
     </row>
     <row r="11" spans="1:21">
-      <c r="A11" s="34" t="s">
+      <c r="A11" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="35"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
-      <c r="J11" s="26"/>
-      <c r="K11" s="26"/>
-      <c r="L11" s="26"/>
-      <c r="M11" s="26"/>
-      <c r="N11" s="26"/>
-      <c r="O11" s="26"/>
-      <c r="P11" s="26"/>
-      <c r="Q11" s="26"/>
-      <c r="R11" s="26"/>
-      <c r="S11" s="26"/>
-      <c r="T11" s="26"/>
-      <c r="U11" s="27"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="27"/>
+      <c r="K11" s="27"/>
+      <c r="L11" s="27"/>
+      <c r="M11" s="27"/>
+      <c r="N11" s="27"/>
+      <c r="O11" s="27"/>
+      <c r="P11" s="27"/>
+      <c r="Q11" s="27"/>
+      <c r="R11" s="27"/>
+      <c r="S11" s="27"/>
+      <c r="T11" s="27"/>
+      <c r="U11" s="36"/>
     </row>
     <row r="12" spans="1:21">
-      <c r="A12" s="34" t="s">
+      <c r="A12" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
-      <c r="J12" s="26"/>
-      <c r="K12" s="26"/>
-      <c r="L12" s="26"/>
-      <c r="M12" s="26"/>
-      <c r="N12" s="26"/>
-      <c r="O12" s="26"/>
-      <c r="P12" s="26"/>
-      <c r="Q12" s="26"/>
-      <c r="R12" s="26"/>
-      <c r="S12" s="26"/>
-      <c r="T12" s="26"/>
-      <c r="U12" s="27"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="27"/>
+      <c r="K12" s="27"/>
+      <c r="L12" s="27"/>
+      <c r="M12" s="27"/>
+      <c r="N12" s="27"/>
+      <c r="O12" s="27"/>
+      <c r="P12" s="27"/>
+      <c r="Q12" s="27"/>
+      <c r="R12" s="27"/>
+      <c r="S12" s="27"/>
+      <c r="T12" s="27"/>
+      <c r="U12" s="36"/>
     </row>
     <row r="13" spans="1:21">
-      <c r="A13" s="34" t="s">
+      <c r="A13" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
-      <c r="J13" s="26"/>
-      <c r="K13" s="26"/>
-      <c r="L13" s="26"/>
-      <c r="M13" s="26"/>
-      <c r="N13" s="26"/>
-      <c r="O13" s="26"/>
-      <c r="P13" s="26"/>
-      <c r="Q13" s="26"/>
-      <c r="R13" s="26"/>
-      <c r="S13" s="26"/>
-      <c r="T13" s="26"/>
-      <c r="U13" s="27"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="27"/>
+      <c r="K13" s="27"/>
+      <c r="L13" s="27"/>
+      <c r="M13" s="27"/>
+      <c r="N13" s="27"/>
+      <c r="O13" s="27"/>
+      <c r="P13" s="27"/>
+      <c r="Q13" s="27"/>
+      <c r="R13" s="27"/>
+      <c r="S13" s="27"/>
+      <c r="T13" s="27"/>
+      <c r="U13" s="36"/>
     </row>
     <row r="14" spans="1:21">
-      <c r="A14" s="34" t="s">
+      <c r="A14" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="35"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="30"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="32"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="31"/>
-      <c r="I14" s="32"/>
-      <c r="J14" s="30"/>
-      <c r="K14" s="31"/>
-      <c r="L14" s="32"/>
-      <c r="M14" s="30"/>
-      <c r="N14" s="31"/>
-      <c r="O14" s="32"/>
-      <c r="P14" s="30"/>
-      <c r="Q14" s="31"/>
-      <c r="R14" s="32"/>
-      <c r="S14" s="30"/>
-      <c r="T14" s="31"/>
-      <c r="U14" s="33"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="40"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="38"/>
+      <c r="I14" s="40"/>
+      <c r="J14" s="37"/>
+      <c r="K14" s="38"/>
+      <c r="L14" s="40"/>
+      <c r="M14" s="37"/>
+      <c r="N14" s="38"/>
+      <c r="O14" s="40"/>
+      <c r="P14" s="37"/>
+      <c r="Q14" s="38"/>
+      <c r="R14" s="40"/>
+      <c r="S14" s="37"/>
+      <c r="T14" s="38"/>
+      <c r="U14" s="39"/>
     </row>
     <row r="15" spans="1:21">
       <c r="A15" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D15" s="26"/>
-      <c r="E15" s="26"/>
-      <c r="F15" s="26"/>
-      <c r="G15" s="26"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="26"/>
-      <c r="J15" s="26"/>
-      <c r="K15" s="26"/>
-      <c r="L15" s="26"/>
-      <c r="M15" s="26"/>
-      <c r="N15" s="26"/>
-      <c r="O15" s="26"/>
-      <c r="P15" s="26"/>
-      <c r="Q15" s="26"/>
-      <c r="R15" s="26"/>
-      <c r="S15" s="26"/>
-      <c r="T15" s="26"/>
-      <c r="U15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="27"/>
+      <c r="L15" s="27"/>
+      <c r="M15" s="27"/>
+      <c r="N15" s="27"/>
+      <c r="O15" s="27"/>
+      <c r="P15" s="27"/>
+      <c r="Q15" s="27"/>
+      <c r="R15" s="27"/>
+      <c r="S15" s="27"/>
+      <c r="T15" s="27"/>
+      <c r="U15" s="36"/>
     </row>
     <row r="16" spans="1:21">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="39"/>
-      <c r="C16" s="39"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
       <c r="D16" s="12" t="s">
         <v>8</v>
       </c>
@@ -1381,159 +1378,159 @@
       </c>
     </row>
     <row r="17" spans="1:21">
-      <c r="A17" s="34" t="s">
+      <c r="A17" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="35"/>
-      <c r="C17" s="35"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="36"/>
-      <c r="F17" s="36"/>
-      <c r="G17" s="36"/>
-      <c r="H17" s="36"/>
-      <c r="I17" s="36"/>
-      <c r="J17" s="36"/>
-      <c r="K17" s="36"/>
-      <c r="L17" s="36"/>
-      <c r="M17" s="36"/>
-      <c r="N17" s="36"/>
-      <c r="O17" s="36"/>
-      <c r="P17" s="36"/>
-      <c r="Q17" s="36"/>
-      <c r="R17" s="36"/>
-      <c r="S17" s="36"/>
-      <c r="T17" s="36"/>
-      <c r="U17" s="37"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="23"/>
+      <c r="K17" s="23"/>
+      <c r="L17" s="23"/>
+      <c r="M17" s="23"/>
+      <c r="N17" s="23"/>
+      <c r="O17" s="23"/>
+      <c r="P17" s="23"/>
+      <c r="Q17" s="23"/>
+      <c r="R17" s="23"/>
+      <c r="S17" s="23"/>
+      <c r="T17" s="23"/>
+      <c r="U17" s="35"/>
     </row>
     <row r="18" spans="1:21">
-      <c r="A18" s="34" t="s">
+      <c r="A18" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="35"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="26"/>
-      <c r="J18" s="26"/>
-      <c r="K18" s="26"/>
-      <c r="L18" s="26"/>
-      <c r="M18" s="26"/>
-      <c r="N18" s="26"/>
-      <c r="O18" s="26"/>
-      <c r="P18" s="26"/>
-      <c r="Q18" s="26"/>
-      <c r="R18" s="26"/>
-      <c r="S18" s="26"/>
-      <c r="T18" s="26"/>
-      <c r="U18" s="27"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="27"/>
+      <c r="J18" s="27"/>
+      <c r="K18" s="27"/>
+      <c r="L18" s="27"/>
+      <c r="M18" s="27"/>
+      <c r="N18" s="27"/>
+      <c r="O18" s="27"/>
+      <c r="P18" s="27"/>
+      <c r="Q18" s="27"/>
+      <c r="R18" s="27"/>
+      <c r="S18" s="27"/>
+      <c r="T18" s="27"/>
+      <c r="U18" s="36"/>
     </row>
     <row r="19" spans="1:21">
-      <c r="A19" s="34" t="s">
+      <c r="A19" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="35"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
-      <c r="J19" s="26"/>
-      <c r="K19" s="26"/>
-      <c r="L19" s="26"/>
-      <c r="M19" s="26"/>
-      <c r="N19" s="26"/>
-      <c r="O19" s="26"/>
-      <c r="P19" s="26"/>
-      <c r="Q19" s="26"/>
-      <c r="R19" s="26"/>
-      <c r="S19" s="26"/>
-      <c r="T19" s="26"/>
-      <c r="U19" s="27"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="27"/>
+      <c r="K19" s="27"/>
+      <c r="L19" s="27"/>
+      <c r="M19" s="27"/>
+      <c r="N19" s="27"/>
+      <c r="O19" s="27"/>
+      <c r="P19" s="27"/>
+      <c r="Q19" s="27"/>
+      <c r="R19" s="27"/>
+      <c r="S19" s="27"/>
+      <c r="T19" s="27"/>
+      <c r="U19" s="36"/>
     </row>
     <row r="20" spans="1:21">
-      <c r="A20" s="34" t="s">
+      <c r="A20" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="35"/>
-      <c r="C20" s="35"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
-      <c r="I20" s="26"/>
-      <c r="J20" s="26"/>
-      <c r="K20" s="26"/>
-      <c r="L20" s="26"/>
-      <c r="M20" s="26"/>
-      <c r="N20" s="26"/>
-      <c r="O20" s="26"/>
-      <c r="P20" s="26"/>
-      <c r="Q20" s="26"/>
-      <c r="R20" s="26"/>
-      <c r="S20" s="26"/>
-      <c r="T20" s="26"/>
-      <c r="U20" s="27"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="27"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="27"/>
+      <c r="K20" s="27"/>
+      <c r="L20" s="27"/>
+      <c r="M20" s="27"/>
+      <c r="N20" s="27"/>
+      <c r="O20" s="27"/>
+      <c r="P20" s="27"/>
+      <c r="Q20" s="27"/>
+      <c r="R20" s="27"/>
+      <c r="S20" s="27"/>
+      <c r="T20" s="27"/>
+      <c r="U20" s="36"/>
     </row>
     <row r="21" spans="1:21">
-      <c r="A21" s="34" t="s">
+      <c r="A21" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="35"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="30"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="31"/>
-      <c r="I21" s="32"/>
-      <c r="J21" s="30"/>
-      <c r="K21" s="31"/>
-      <c r="L21" s="32"/>
-      <c r="M21" s="30"/>
-      <c r="N21" s="31"/>
-      <c r="O21" s="32"/>
-      <c r="P21" s="30"/>
-      <c r="Q21" s="31"/>
-      <c r="R21" s="32"/>
-      <c r="S21" s="30"/>
-      <c r="T21" s="31"/>
-      <c r="U21" s="33"/>
+      <c r="B21" s="22"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="38"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="38"/>
+      <c r="I21" s="40"/>
+      <c r="J21" s="37"/>
+      <c r="K21" s="38"/>
+      <c r="L21" s="40"/>
+      <c r="M21" s="37"/>
+      <c r="N21" s="38"/>
+      <c r="O21" s="40"/>
+      <c r="P21" s="37"/>
+      <c r="Q21" s="38"/>
+      <c r="R21" s="40"/>
+      <c r="S21" s="37"/>
+      <c r="T21" s="38"/>
+      <c r="U21" s="39"/>
     </row>
     <row r="22" spans="1:21">
       <c r="A22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="26"/>
-      <c r="G22" s="26"/>
-      <c r="H22" s="26"/>
-      <c r="I22" s="26"/>
-      <c r="J22" s="26"/>
-      <c r="K22" s="26"/>
-      <c r="L22" s="26"/>
-      <c r="M22" s="26"/>
-      <c r="N22" s="26"/>
-      <c r="O22" s="26"/>
-      <c r="P22" s="26"/>
-      <c r="Q22" s="26"/>
-      <c r="R22" s="26"/>
-      <c r="S22" s="26"/>
-      <c r="T22" s="26"/>
-      <c r="U22" s="27"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="27"/>
+      <c r="I22" s="27"/>
+      <c r="J22" s="27"/>
+      <c r="K22" s="27"/>
+      <c r="L22" s="27"/>
+      <c r="M22" s="27"/>
+      <c r="N22" s="27"/>
+      <c r="O22" s="27"/>
+      <c r="P22" s="27"/>
+      <c r="Q22" s="27"/>
+      <c r="R22" s="27"/>
+      <c r="S22" s="27"/>
+      <c r="T22" s="27"/>
+      <c r="U22" s="36"/>
     </row>
     <row r="23" spans="1:21">
-      <c r="A23" s="38" t="s">
+      <c r="A23" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B23" s="39"/>
-      <c r="C23" s="39"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
       <c r="D23" s="12" t="s">
         <v>8</v>
       </c>
@@ -1590,159 +1587,159 @@
       </c>
     </row>
     <row r="24" spans="1:21">
-      <c r="A24" s="34" t="s">
+      <c r="A24" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B24" s="35"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="36"/>
-      <c r="H24" s="36"/>
-      <c r="I24" s="36"/>
-      <c r="J24" s="36"/>
-      <c r="K24" s="36"/>
-      <c r="L24" s="36"/>
-      <c r="M24" s="36"/>
-      <c r="N24" s="36"/>
-      <c r="O24" s="36"/>
-      <c r="P24" s="36"/>
-      <c r="Q24" s="36"/>
-      <c r="R24" s="36"/>
-      <c r="S24" s="36"/>
-      <c r="T24" s="36"/>
-      <c r="U24" s="37"/>
+      <c r="B24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="23"/>
+      <c r="H24" s="23"/>
+      <c r="I24" s="23"/>
+      <c r="J24" s="23"/>
+      <c r="K24" s="23"/>
+      <c r="L24" s="23"/>
+      <c r="M24" s="23"/>
+      <c r="N24" s="23"/>
+      <c r="O24" s="23"/>
+      <c r="P24" s="23"/>
+      <c r="Q24" s="23"/>
+      <c r="R24" s="23"/>
+      <c r="S24" s="23"/>
+      <c r="T24" s="23"/>
+      <c r="U24" s="35"/>
     </row>
     <row r="25" spans="1:21">
-      <c r="A25" s="34" t="s">
+      <c r="A25" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B25" s="35"/>
-      <c r="C25" s="35"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="26"/>
-      <c r="F25" s="26"/>
-      <c r="G25" s="26"/>
-      <c r="H25" s="26"/>
-      <c r="I25" s="26"/>
-      <c r="J25" s="26"/>
-      <c r="K25" s="26"/>
-      <c r="L25" s="26"/>
-      <c r="M25" s="26"/>
-      <c r="N25" s="26"/>
-      <c r="O25" s="26"/>
-      <c r="P25" s="26"/>
-      <c r="Q25" s="26"/>
-      <c r="R25" s="26"/>
-      <c r="S25" s="26"/>
-      <c r="T25" s="26"/>
-      <c r="U25" s="27"/>
+      <c r="B25" s="22"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="27"/>
+      <c r="I25" s="27"/>
+      <c r="J25" s="27"/>
+      <c r="K25" s="27"/>
+      <c r="L25" s="27"/>
+      <c r="M25" s="27"/>
+      <c r="N25" s="27"/>
+      <c r="O25" s="27"/>
+      <c r="P25" s="27"/>
+      <c r="Q25" s="27"/>
+      <c r="R25" s="27"/>
+      <c r="S25" s="27"/>
+      <c r="T25" s="27"/>
+      <c r="U25" s="36"/>
     </row>
     <row r="26" spans="1:21">
-      <c r="A26" s="34" t="s">
+      <c r="A26" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B26" s="35"/>
-      <c r="C26" s="35"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="26"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="26"/>
-      <c r="H26" s="26"/>
-      <c r="I26" s="26"/>
-      <c r="J26" s="26"/>
-      <c r="K26" s="26"/>
-      <c r="L26" s="26"/>
-      <c r="M26" s="26"/>
-      <c r="N26" s="26"/>
-      <c r="O26" s="26"/>
-      <c r="P26" s="26"/>
-      <c r="Q26" s="26"/>
-      <c r="R26" s="26"/>
-      <c r="S26" s="26"/>
-      <c r="T26" s="26"/>
-      <c r="U26" s="27"/>
+      <c r="B26" s="22"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="27"/>
+      <c r="H26" s="27"/>
+      <c r="I26" s="27"/>
+      <c r="J26" s="27"/>
+      <c r="K26" s="27"/>
+      <c r="L26" s="27"/>
+      <c r="M26" s="27"/>
+      <c r="N26" s="27"/>
+      <c r="O26" s="27"/>
+      <c r="P26" s="27"/>
+      <c r="Q26" s="27"/>
+      <c r="R26" s="27"/>
+      <c r="S26" s="27"/>
+      <c r="T26" s="27"/>
+      <c r="U26" s="36"/>
     </row>
     <row r="27" spans="1:21">
-      <c r="A27" s="34" t="s">
+      <c r="A27" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="B27" s="35"/>
-      <c r="C27" s="35"/>
-      <c r="D27" s="26"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="26"/>
-      <c r="H27" s="26"/>
-      <c r="I27" s="26"/>
-      <c r="J27" s="26"/>
-      <c r="K27" s="26"/>
-      <c r="L27" s="26"/>
-      <c r="M27" s="26"/>
-      <c r="N27" s="26"/>
-      <c r="O27" s="26"/>
-      <c r="P27" s="26"/>
-      <c r="Q27" s="26"/>
-      <c r="R27" s="26"/>
-      <c r="S27" s="26"/>
-      <c r="T27" s="26"/>
-      <c r="U27" s="27"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="27"/>
+      <c r="I27" s="27"/>
+      <c r="J27" s="27"/>
+      <c r="K27" s="27"/>
+      <c r="L27" s="27"/>
+      <c r="M27" s="27"/>
+      <c r="N27" s="27"/>
+      <c r="O27" s="27"/>
+      <c r="P27" s="27"/>
+      <c r="Q27" s="27"/>
+      <c r="R27" s="27"/>
+      <c r="S27" s="27"/>
+      <c r="T27" s="27"/>
+      <c r="U27" s="36"/>
     </row>
     <row r="28" spans="1:21">
-      <c r="A28" s="34" t="s">
+      <c r="A28" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B28" s="35"/>
-      <c r="C28" s="35"/>
-      <c r="D28" s="30"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="31"/>
-      <c r="I28" s="32"/>
-      <c r="J28" s="30"/>
-      <c r="K28" s="31"/>
-      <c r="L28" s="32"/>
-      <c r="M28" s="30"/>
-      <c r="N28" s="31"/>
-      <c r="O28" s="32"/>
-      <c r="P28" s="30"/>
-      <c r="Q28" s="31"/>
-      <c r="R28" s="32"/>
-      <c r="S28" s="30"/>
-      <c r="T28" s="31"/>
-      <c r="U28" s="33"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="37"/>
+      <c r="H28" s="38"/>
+      <c r="I28" s="40"/>
+      <c r="J28" s="37"/>
+      <c r="K28" s="38"/>
+      <c r="L28" s="40"/>
+      <c r="M28" s="37"/>
+      <c r="N28" s="38"/>
+      <c r="O28" s="40"/>
+      <c r="P28" s="37"/>
+      <c r="Q28" s="38"/>
+      <c r="R28" s="40"/>
+      <c r="S28" s="37"/>
+      <c r="T28" s="38"/>
+      <c r="U28" s="39"/>
     </row>
     <row r="29" spans="1:21">
       <c r="A29" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D29" s="26"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26"/>
-      <c r="H29" s="26"/>
-      <c r="I29" s="26"/>
-      <c r="J29" s="26"/>
-      <c r="K29" s="26"/>
-      <c r="L29" s="26"/>
-      <c r="M29" s="26"/>
-      <c r="N29" s="26"/>
-      <c r="O29" s="26"/>
-      <c r="P29" s="26"/>
-      <c r="Q29" s="26"/>
-      <c r="R29" s="26"/>
-      <c r="S29" s="26"/>
-      <c r="T29" s="26"/>
-      <c r="U29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="27"/>
+      <c r="G29" s="27"/>
+      <c r="H29" s="27"/>
+      <c r="I29" s="27"/>
+      <c r="J29" s="27"/>
+      <c r="K29" s="27"/>
+      <c r="L29" s="27"/>
+      <c r="M29" s="27"/>
+      <c r="N29" s="27"/>
+      <c r="O29" s="27"/>
+      <c r="P29" s="27"/>
+      <c r="Q29" s="27"/>
+      <c r="R29" s="27"/>
+      <c r="S29" s="27"/>
+      <c r="T29" s="27"/>
+      <c r="U29" s="36"/>
     </row>
     <row r="30" spans="1:21">
-      <c r="A30" s="38" t="s">
+      <c r="A30" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B30" s="39"/>
-      <c r="C30" s="39"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
       <c r="D30" s="12" t="s">
         <v>8</v>
       </c>
@@ -1799,154 +1796,154 @@
       </c>
     </row>
     <row r="31" spans="1:21">
-      <c r="A31" s="34" t="s">
+      <c r="A31" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B31" s="35"/>
-      <c r="C31" s="35"/>
-      <c r="D31" s="36"/>
-      <c r="E31" s="36"/>
-      <c r="F31" s="36"/>
-      <c r="G31" s="36"/>
-      <c r="H31" s="36"/>
-      <c r="I31" s="36"/>
-      <c r="J31" s="36"/>
-      <c r="K31" s="36"/>
-      <c r="L31" s="36"/>
-      <c r="M31" s="36"/>
-      <c r="N31" s="36"/>
-      <c r="O31" s="36"/>
-      <c r="P31" s="36"/>
-      <c r="Q31" s="36"/>
-      <c r="R31" s="36"/>
-      <c r="S31" s="36"/>
-      <c r="T31" s="36"/>
-      <c r="U31" s="37"/>
+      <c r="B31" s="22"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="23"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="23"/>
+      <c r="H31" s="23"/>
+      <c r="I31" s="23"/>
+      <c r="J31" s="23"/>
+      <c r="K31" s="23"/>
+      <c r="L31" s="23"/>
+      <c r="M31" s="23"/>
+      <c r="N31" s="23"/>
+      <c r="O31" s="23"/>
+      <c r="P31" s="23"/>
+      <c r="Q31" s="23"/>
+      <c r="R31" s="23"/>
+      <c r="S31" s="23"/>
+      <c r="T31" s="23"/>
+      <c r="U31" s="35"/>
     </row>
     <row r="32" spans="1:21">
-      <c r="A32" s="34" t="s">
+      <c r="A32" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B32" s="35"/>
-      <c r="C32" s="35"/>
-      <c r="D32" s="26"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="26"/>
-      <c r="I32" s="26"/>
-      <c r="J32" s="26"/>
-      <c r="K32" s="26"/>
-      <c r="L32" s="26"/>
-      <c r="M32" s="26"/>
-      <c r="N32" s="26"/>
-      <c r="O32" s="26"/>
-      <c r="P32" s="26"/>
-      <c r="Q32" s="26"/>
-      <c r="R32" s="26"/>
-      <c r="S32" s="26"/>
-      <c r="T32" s="26"/>
-      <c r="U32" s="27"/>
+      <c r="B32" s="22"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="27"/>
+      <c r="F32" s="27"/>
+      <c r="G32" s="27"/>
+      <c r="H32" s="27"/>
+      <c r="I32" s="27"/>
+      <c r="J32" s="27"/>
+      <c r="K32" s="27"/>
+      <c r="L32" s="27"/>
+      <c r="M32" s="27"/>
+      <c r="N32" s="27"/>
+      <c r="O32" s="27"/>
+      <c r="P32" s="27"/>
+      <c r="Q32" s="27"/>
+      <c r="R32" s="27"/>
+      <c r="S32" s="27"/>
+      <c r="T32" s="27"/>
+      <c r="U32" s="36"/>
     </row>
     <row r="33" spans="1:21">
-      <c r="A33" s="34" t="s">
+      <c r="A33" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B33" s="35"/>
-      <c r="C33" s="35"/>
-      <c r="D33" s="26"/>
-      <c r="E33" s="26"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="26"/>
-      <c r="I33" s="26"/>
-      <c r="J33" s="26"/>
-      <c r="K33" s="26"/>
-      <c r="L33" s="26"/>
-      <c r="M33" s="26"/>
-      <c r="N33" s="26"/>
-      <c r="O33" s="26"/>
-      <c r="P33" s="26"/>
-      <c r="Q33" s="26"/>
-      <c r="R33" s="26"/>
-      <c r="S33" s="26"/>
-      <c r="T33" s="26"/>
-      <c r="U33" s="27"/>
+      <c r="B33" s="22"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="27"/>
+      <c r="G33" s="27"/>
+      <c r="H33" s="27"/>
+      <c r="I33" s="27"/>
+      <c r="J33" s="27"/>
+      <c r="K33" s="27"/>
+      <c r="L33" s="27"/>
+      <c r="M33" s="27"/>
+      <c r="N33" s="27"/>
+      <c r="O33" s="27"/>
+      <c r="P33" s="27"/>
+      <c r="Q33" s="27"/>
+      <c r="R33" s="27"/>
+      <c r="S33" s="27"/>
+      <c r="T33" s="27"/>
+      <c r="U33" s="36"/>
     </row>
     <row r="34" spans="1:21">
-      <c r="A34" s="34" t="s">
+      <c r="A34" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="B34" s="35"/>
-      <c r="C34" s="35"/>
-      <c r="D34" s="26"/>
-      <c r="E34" s="26"/>
-      <c r="F34" s="26"/>
-      <c r="G34" s="26"/>
-      <c r="H34" s="26"/>
-      <c r="I34" s="26"/>
-      <c r="J34" s="26"/>
-      <c r="K34" s="26"/>
-      <c r="L34" s="26"/>
-      <c r="M34" s="26"/>
-      <c r="N34" s="26"/>
-      <c r="O34" s="26"/>
-      <c r="P34" s="26"/>
-      <c r="Q34" s="26"/>
-      <c r="R34" s="26"/>
-      <c r="S34" s="26"/>
-      <c r="T34" s="26"/>
-      <c r="U34" s="27"/>
+      <c r="B34" s="22"/>
+      <c r="C34" s="22"/>
+      <c r="D34" s="27"/>
+      <c r="E34" s="27"/>
+      <c r="F34" s="27"/>
+      <c r="G34" s="27"/>
+      <c r="H34" s="27"/>
+      <c r="I34" s="27"/>
+      <c r="J34" s="27"/>
+      <c r="K34" s="27"/>
+      <c r="L34" s="27"/>
+      <c r="M34" s="27"/>
+      <c r="N34" s="27"/>
+      <c r="O34" s="27"/>
+      <c r="P34" s="27"/>
+      <c r="Q34" s="27"/>
+      <c r="R34" s="27"/>
+      <c r="S34" s="27"/>
+      <c r="T34" s="27"/>
+      <c r="U34" s="36"/>
     </row>
     <row r="35" spans="1:21">
-      <c r="A35" s="34" t="s">
+      <c r="A35" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B35" s="35"/>
-      <c r="C35" s="35"/>
-      <c r="D35" s="26"/>
-      <c r="E35" s="26"/>
-      <c r="F35" s="26"/>
-      <c r="G35" s="26"/>
-      <c r="H35" s="26"/>
-      <c r="I35" s="26"/>
-      <c r="J35" s="26"/>
-      <c r="K35" s="26"/>
-      <c r="L35" s="26"/>
-      <c r="M35" s="26"/>
-      <c r="N35" s="26"/>
-      <c r="O35" s="26"/>
-      <c r="P35" s="26"/>
-      <c r="Q35" s="26"/>
-      <c r="R35" s="26"/>
-      <c r="S35" s="26"/>
-      <c r="T35" s="26"/>
-      <c r="U35" s="27"/>
+      <c r="B35" s="22"/>
+      <c r="C35" s="22"/>
+      <c r="D35" s="27"/>
+      <c r="E35" s="27"/>
+      <c r="F35" s="27"/>
+      <c r="G35" s="27"/>
+      <c r="H35" s="27"/>
+      <c r="I35" s="27"/>
+      <c r="J35" s="27"/>
+      <c r="K35" s="27"/>
+      <c r="L35" s="27"/>
+      <c r="M35" s="27"/>
+      <c r="N35" s="27"/>
+      <c r="O35" s="27"/>
+      <c r="P35" s="27"/>
+      <c r="Q35" s="27"/>
+      <c r="R35" s="27"/>
+      <c r="S35" s="27"/>
+      <c r="T35" s="27"/>
+      <c r="U35" s="36"/>
     </row>
     <row r="36" spans="1:21">
-      <c r="A36" s="28" t="s">
+      <c r="A36" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="B36" s="29"/>
-      <c r="C36" s="29"/>
-      <c r="D36" s="30"/>
-      <c r="E36" s="31"/>
-      <c r="F36" s="32"/>
-      <c r="G36" s="30"/>
-      <c r="H36" s="31"/>
-      <c r="I36" s="32"/>
-      <c r="J36" s="30"/>
-      <c r="K36" s="31"/>
-      <c r="L36" s="32"/>
-      <c r="M36" s="30"/>
-      <c r="N36" s="31"/>
-      <c r="O36" s="32"/>
-      <c r="P36" s="30"/>
-      <c r="Q36" s="31"/>
-      <c r="R36" s="32"/>
-      <c r="S36" s="30"/>
-      <c r="T36" s="31"/>
-      <c r="U36" s="33"/>
+      <c r="B36" s="46"/>
+      <c r="C36" s="46"/>
+      <c r="D36" s="37"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="40"/>
+      <c r="G36" s="37"/>
+      <c r="H36" s="38"/>
+      <c r="I36" s="40"/>
+      <c r="J36" s="37"/>
+      <c r="K36" s="38"/>
+      <c r="L36" s="40"/>
+      <c r="M36" s="37"/>
+      <c r="N36" s="38"/>
+      <c r="O36" s="40"/>
+      <c r="P36" s="37"/>
+      <c r="Q36" s="38"/>
+      <c r="R36" s="40"/>
+      <c r="S36" s="37"/>
+      <c r="T36" s="38"/>
+      <c r="U36" s="39"/>
     </row>
     <row r="37" spans="1:21">
       <c r="A37" s="1"/>
@@ -2009,98 +2006,98 @@
       <c r="U42" s="3"/>
     </row>
     <row r="43" spans="1:21">
-      <c r="A43" s="17" t="s">
+      <c r="A43" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="B43" s="18"/>
-      <c r="C43" s="18"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="18"/>
-      <c r="F43" s="18"/>
-      <c r="G43" s="18"/>
-      <c r="H43" s="18"/>
-      <c r="I43" s="18"/>
-      <c r="J43" s="18"/>
-      <c r="K43" s="18"/>
-      <c r="L43" s="18"/>
-      <c r="M43" s="18"/>
-      <c r="N43" s="18"/>
-      <c r="O43" s="18"/>
-      <c r="P43" s="18"/>
-      <c r="Q43" s="18"/>
-      <c r="R43" s="18"/>
-      <c r="S43" s="18"/>
-      <c r="T43" s="18"/>
-      <c r="U43" s="19"/>
+      <c r="B43" s="48"/>
+      <c r="C43" s="48"/>
+      <c r="D43" s="48"/>
+      <c r="E43" s="48"/>
+      <c r="F43" s="48"/>
+      <c r="G43" s="48"/>
+      <c r="H43" s="48"/>
+      <c r="I43" s="48"/>
+      <c r="J43" s="48"/>
+      <c r="K43" s="48"/>
+      <c r="L43" s="48"/>
+      <c r="M43" s="48"/>
+      <c r="N43" s="48"/>
+      <c r="O43" s="48"/>
+      <c r="P43" s="48"/>
+      <c r="Q43" s="48"/>
+      <c r="R43" s="48"/>
+      <c r="S43" s="48"/>
+      <c r="T43" s="48"/>
+      <c r="U43" s="49"/>
     </row>
     <row r="44" spans="1:21">
-      <c r="A44" s="17"/>
-      <c r="B44" s="18"/>
-      <c r="C44" s="18"/>
-      <c r="D44" s="18"/>
-      <c r="E44" s="18"/>
-      <c r="F44" s="18"/>
-      <c r="G44" s="18"/>
-      <c r="H44" s="18"/>
-      <c r="I44" s="18"/>
-      <c r="J44" s="18"/>
-      <c r="K44" s="18"/>
-      <c r="L44" s="18"/>
-      <c r="M44" s="18"/>
-      <c r="N44" s="18"/>
-      <c r="O44" s="18"/>
-      <c r="P44" s="18"/>
-      <c r="Q44" s="18"/>
-      <c r="R44" s="18"/>
-      <c r="S44" s="18"/>
-      <c r="T44" s="18"/>
-      <c r="U44" s="19"/>
+      <c r="A44" s="47"/>
+      <c r="B44" s="48"/>
+      <c r="C44" s="48"/>
+      <c r="D44" s="48"/>
+      <c r="E44" s="48"/>
+      <c r="F44" s="48"/>
+      <c r="G44" s="48"/>
+      <c r="H44" s="48"/>
+      <c r="I44" s="48"/>
+      <c r="J44" s="48"/>
+      <c r="K44" s="48"/>
+      <c r="L44" s="48"/>
+      <c r="M44" s="48"/>
+      <c r="N44" s="48"/>
+      <c r="O44" s="48"/>
+      <c r="P44" s="48"/>
+      <c r="Q44" s="48"/>
+      <c r="R44" s="48"/>
+      <c r="S44" s="48"/>
+      <c r="T44" s="48"/>
+      <c r="U44" s="49"/>
     </row>
     <row r="45" spans="1:21">
-      <c r="A45" s="17"/>
-      <c r="B45" s="18"/>
-      <c r="C45" s="18"/>
-      <c r="D45" s="18"/>
-      <c r="E45" s="18"/>
-      <c r="F45" s="18"/>
-      <c r="G45" s="18"/>
-      <c r="H45" s="18"/>
-      <c r="I45" s="18"/>
-      <c r="J45" s="18"/>
-      <c r="K45" s="18"/>
-      <c r="L45" s="18"/>
-      <c r="M45" s="18"/>
-      <c r="N45" s="18"/>
-      <c r="O45" s="18"/>
-      <c r="P45" s="18"/>
-      <c r="Q45" s="18"/>
-      <c r="R45" s="18"/>
-      <c r="S45" s="18"/>
-      <c r="T45" s="18"/>
-      <c r="U45" s="19"/>
+      <c r="A45" s="47"/>
+      <c r="B45" s="48"/>
+      <c r="C45" s="48"/>
+      <c r="D45" s="48"/>
+      <c r="E45" s="48"/>
+      <c r="F45" s="48"/>
+      <c r="G45" s="48"/>
+      <c r="H45" s="48"/>
+      <c r="I45" s="48"/>
+      <c r="J45" s="48"/>
+      <c r="K45" s="48"/>
+      <c r="L45" s="48"/>
+      <c r="M45" s="48"/>
+      <c r="N45" s="48"/>
+      <c r="O45" s="48"/>
+      <c r="P45" s="48"/>
+      <c r="Q45" s="48"/>
+      <c r="R45" s="48"/>
+      <c r="S45" s="48"/>
+      <c r="T45" s="48"/>
+      <c r="U45" s="49"/>
     </row>
     <row r="46" spans="1:21">
-      <c r="A46" s="17"/>
-      <c r="B46" s="18"/>
-      <c r="C46" s="18"/>
-      <c r="D46" s="18"/>
-      <c r="E46" s="18"/>
-      <c r="F46" s="18"/>
-      <c r="G46" s="18"/>
-      <c r="H46" s="18"/>
-      <c r="I46" s="18"/>
-      <c r="J46" s="18"/>
-      <c r="K46" s="18"/>
-      <c r="L46" s="18"/>
-      <c r="M46" s="18"/>
-      <c r="N46" s="18"/>
-      <c r="O46" s="18"/>
-      <c r="P46" s="18"/>
-      <c r="Q46" s="18"/>
-      <c r="R46" s="18"/>
-      <c r="S46" s="18"/>
-      <c r="T46" s="18"/>
-      <c r="U46" s="19"/>
+      <c r="A46" s="47"/>
+      <c r="B46" s="48"/>
+      <c r="C46" s="48"/>
+      <c r="D46" s="48"/>
+      <c r="E46" s="48"/>
+      <c r="F46" s="48"/>
+      <c r="G46" s="48"/>
+      <c r="H46" s="48"/>
+      <c r="I46" s="48"/>
+      <c r="J46" s="48"/>
+      <c r="K46" s="48"/>
+      <c r="L46" s="48"/>
+      <c r="M46" s="48"/>
+      <c r="N46" s="48"/>
+      <c r="O46" s="48"/>
+      <c r="P46" s="48"/>
+      <c r="Q46" s="48"/>
+      <c r="R46" s="48"/>
+      <c r="S46" s="48"/>
+      <c r="T46" s="48"/>
+      <c r="U46" s="49"/>
     </row>
     <row r="47" spans="1:21">
       <c r="A47" s="1"/>
@@ -2111,107 +2108,270 @@
       <c r="U48" s="3"/>
     </row>
     <row r="49" spans="1:21">
-      <c r="A49" s="20" t="s">
+      <c r="A49" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="B49" s="21"/>
-      <c r="C49" s="21"/>
-      <c r="D49" s="21"/>
-      <c r="J49" s="21" t="s">
+      <c r="B49" s="17"/>
+      <c r="C49" s="17"/>
+      <c r="D49" s="17"/>
+      <c r="J49" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="K49" s="21"/>
-      <c r="L49" s="21"/>
-      <c r="M49" s="21"/>
-      <c r="R49" s="21" t="s">
+      <c r="K49" s="17"/>
+      <c r="L49" s="17"/>
+      <c r="M49" s="17"/>
+      <c r="R49" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="S49" s="21"/>
-      <c r="T49" s="21"/>
-      <c r="U49" s="22"/>
+      <c r="S49" s="17"/>
+      <c r="T49" s="17"/>
+      <c r="U49" s="18"/>
     </row>
     <row r="50" spans="1:21">
-      <c r="A50" s="20"/>
-      <c r="B50" s="50"/>
-      <c r="C50" s="50"/>
-      <c r="D50" s="50"/>
-      <c r="J50" s="21"/>
-      <c r="K50" s="21"/>
-      <c r="L50" s="21"/>
-      <c r="M50" s="21"/>
-      <c r="R50" s="21"/>
-      <c r="S50" s="21"/>
-      <c r="T50" s="21"/>
-      <c r="U50" s="22"/>
+      <c r="A50" s="16"/>
+      <c r="B50" s="17"/>
+      <c r="C50" s="17"/>
+      <c r="D50" s="17"/>
+      <c r="J50" s="17"/>
+      <c r="K50" s="17"/>
+      <c r="L50" s="17"/>
+      <c r="M50" s="17"/>
+      <c r="R50" s="17"/>
+      <c r="S50" s="17"/>
+      <c r="T50" s="17"/>
+      <c r="U50" s="18"/>
     </row>
     <row r="51" spans="1:21">
-      <c r="A51" s="20"/>
-      <c r="B51" s="50"/>
-      <c r="C51" s="50"/>
-      <c r="D51" s="50"/>
-      <c r="J51" s="21"/>
-      <c r="K51" s="21"/>
-      <c r="L51" s="21"/>
-      <c r="M51" s="21"/>
-      <c r="R51" s="21"/>
-      <c r="S51" s="21"/>
-      <c r="T51" s="21"/>
-      <c r="U51" s="22"/>
+      <c r="A51" s="16"/>
+      <c r="B51" s="17"/>
+      <c r="C51" s="17"/>
+      <c r="D51" s="17"/>
+      <c r="J51" s="17"/>
+      <c r="K51" s="17"/>
+      <c r="L51" s="17"/>
+      <c r="M51" s="17"/>
+      <c r="R51" s="17"/>
+      <c r="S51" s="17"/>
+      <c r="T51" s="17"/>
+      <c r="U51" s="18"/>
     </row>
     <row r="52" spans="1:21">
-      <c r="A52" s="20"/>
-      <c r="B52" s="50"/>
-      <c r="C52" s="50"/>
-      <c r="D52" s="50"/>
-      <c r="J52" s="21"/>
-      <c r="K52" s="21"/>
-      <c r="L52" s="21"/>
-      <c r="M52" s="21"/>
-      <c r="R52" s="21"/>
-      <c r="S52" s="21"/>
-      <c r="T52" s="21"/>
-      <c r="U52" s="22"/>
+      <c r="A52" s="16"/>
+      <c r="B52" s="17"/>
+      <c r="C52" s="17"/>
+      <c r="D52" s="17"/>
+      <c r="J52" s="17"/>
+      <c r="K52" s="17"/>
+      <c r="L52" s="17"/>
+      <c r="M52" s="17"/>
+      <c r="R52" s="17"/>
+      <c r="S52" s="17"/>
+      <c r="T52" s="17"/>
+      <c r="U52" s="18"/>
     </row>
     <row r="53" spans="1:21" ht="15" thickBot="1">
-      <c r="A53" s="23" t="s">
+      <c r="A53" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="B53" s="24"/>
-      <c r="C53" s="24"/>
-      <c r="D53" s="24"/>
+      <c r="B53" s="43"/>
+      <c r="C53" s="43"/>
+      <c r="D53" s="43"/>
       <c r="E53" s="15"/>
       <c r="F53" s="15"/>
       <c r="G53" s="15"/>
       <c r="H53" s="15"/>
       <c r="I53" s="15"/>
-      <c r="J53" s="24" t="s">
+      <c r="J53" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="K53" s="24"/>
-      <c r="L53" s="24"/>
-      <c r="M53" s="24"/>
+      <c r="K53" s="43"/>
+      <c r="L53" s="43"/>
+      <c r="M53" s="43"/>
       <c r="N53" s="15"/>
       <c r="O53" s="15"/>
       <c r="P53" s="15"/>
       <c r="Q53" s="15"/>
-      <c r="R53" s="24" t="s">
+      <c r="R53" s="43" t="s">
         <v>33</v>
       </c>
-      <c r="S53" s="24"/>
-      <c r="T53" s="24"/>
-      <c r="U53" s="25"/>
+      <c r="S53" s="43"/>
+      <c r="T53" s="43"/>
+      <c r="U53" s="44"/>
     </row>
     <row r="54" spans="1:21" ht="15" thickTop="1">
-      <c r="Q54" s="16" t="s">
+      <c r="Q54" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="R54" s="16"/>
-      <c r="S54" s="16"/>
-      <c r="T54" s="16"/>
-      <c r="U54" s="16"/>
+      <c r="R54" s="41"/>
+      <c r="S54" s="41"/>
+      <c r="T54" s="41"/>
+      <c r="U54" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="187">
+    <mergeCell ref="Q54:U54"/>
+    <mergeCell ref="A43:U46"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="J49:M49"/>
+    <mergeCell ref="R49:U49"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="J53:M53"/>
+    <mergeCell ref="R53:U53"/>
+    <mergeCell ref="S35:U35"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="D36:F36"/>
+    <mergeCell ref="G36:I36"/>
+    <mergeCell ref="J36:L36"/>
+    <mergeCell ref="M36:O36"/>
+    <mergeCell ref="P36:R36"/>
+    <mergeCell ref="S36:U36"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="D35:F35"/>
+    <mergeCell ref="G35:I35"/>
+    <mergeCell ref="J35:L35"/>
+    <mergeCell ref="M35:O35"/>
+    <mergeCell ref="P35:R35"/>
+    <mergeCell ref="J50:M52"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="D32:F32"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="J32:L32"/>
+    <mergeCell ref="M32:O32"/>
+    <mergeCell ref="P32:R32"/>
+    <mergeCell ref="S32:U32"/>
+    <mergeCell ref="S33:U33"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="D34:F34"/>
+    <mergeCell ref="G34:I34"/>
+    <mergeCell ref="J34:L34"/>
+    <mergeCell ref="M34:O34"/>
+    <mergeCell ref="P34:R34"/>
+    <mergeCell ref="S34:U34"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="J33:L33"/>
+    <mergeCell ref="M33:O33"/>
+    <mergeCell ref="P33:R33"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="D31:F31"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="J31:L31"/>
+    <mergeCell ref="M31:O31"/>
+    <mergeCell ref="S28:U28"/>
+    <mergeCell ref="D29:F29"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="J29:L29"/>
+    <mergeCell ref="M29:O29"/>
+    <mergeCell ref="P29:R29"/>
+    <mergeCell ref="S29:U29"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="G28:I28"/>
+    <mergeCell ref="J28:L28"/>
+    <mergeCell ref="M28:O28"/>
+    <mergeCell ref="P28:R28"/>
+    <mergeCell ref="P31:R31"/>
+    <mergeCell ref="S31:U31"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="J25:L25"/>
+    <mergeCell ref="M25:O25"/>
+    <mergeCell ref="P25:R25"/>
+    <mergeCell ref="S25:U25"/>
+    <mergeCell ref="S26:U26"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="J27:L27"/>
+    <mergeCell ref="M27:O27"/>
+    <mergeCell ref="P27:R27"/>
+    <mergeCell ref="S27:U27"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="J26:L26"/>
+    <mergeCell ref="M26:O26"/>
+    <mergeCell ref="P26:R26"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="J24:L24"/>
+    <mergeCell ref="M24:O24"/>
+    <mergeCell ref="S21:U21"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="G22:I22"/>
+    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="M22:O22"/>
+    <mergeCell ref="P22:R22"/>
+    <mergeCell ref="S22:U22"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="J21:L21"/>
+    <mergeCell ref="M21:O21"/>
+    <mergeCell ref="P21:R21"/>
+    <mergeCell ref="P24:R24"/>
+    <mergeCell ref="S24:U24"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="J18:L18"/>
+    <mergeCell ref="M18:O18"/>
+    <mergeCell ref="P18:R18"/>
+    <mergeCell ref="S18:U18"/>
+    <mergeCell ref="S19:U19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="M20:O20"/>
+    <mergeCell ref="P20:R20"/>
+    <mergeCell ref="S20:U20"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="P19:R19"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="M17:O17"/>
+    <mergeCell ref="S14:U14"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="J15:L15"/>
+    <mergeCell ref="M15:O15"/>
+    <mergeCell ref="P15:R15"/>
+    <mergeCell ref="S15:U15"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="M14:O14"/>
+    <mergeCell ref="P14:R14"/>
+    <mergeCell ref="P17:R17"/>
+    <mergeCell ref="S17:U17"/>
+    <mergeCell ref="S12:U12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="M13:O13"/>
+    <mergeCell ref="P13:R13"/>
+    <mergeCell ref="S13:U13"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="J12:L12"/>
+    <mergeCell ref="M12:O12"/>
+    <mergeCell ref="P12:R12"/>
     <mergeCell ref="A50:D52"/>
     <mergeCell ref="R50:U52"/>
     <mergeCell ref="A9:C9"/>
@@ -2236,169 +2396,6 @@
     <mergeCell ref="M11:O11"/>
     <mergeCell ref="P11:R11"/>
     <mergeCell ref="S11:U11"/>
-    <mergeCell ref="S12:U12"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="M13:O13"/>
-    <mergeCell ref="P13:R13"/>
-    <mergeCell ref="S13:U13"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="J12:L12"/>
-    <mergeCell ref="M12:O12"/>
-    <mergeCell ref="P12:R12"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="M17:O17"/>
-    <mergeCell ref="S14:U14"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="J15:L15"/>
-    <mergeCell ref="M15:O15"/>
-    <mergeCell ref="P15:R15"/>
-    <mergeCell ref="S15:U15"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="M14:O14"/>
-    <mergeCell ref="P14:R14"/>
-    <mergeCell ref="P17:R17"/>
-    <mergeCell ref="S17:U17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="J18:L18"/>
-    <mergeCell ref="M18:O18"/>
-    <mergeCell ref="P18:R18"/>
-    <mergeCell ref="S18:U18"/>
-    <mergeCell ref="S19:U19"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="J20:L20"/>
-    <mergeCell ref="M20:O20"/>
-    <mergeCell ref="P20:R20"/>
-    <mergeCell ref="S20:U20"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="P19:R19"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="J24:L24"/>
-    <mergeCell ref="M24:O24"/>
-    <mergeCell ref="S21:U21"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="G22:I22"/>
-    <mergeCell ref="J22:L22"/>
-    <mergeCell ref="M22:O22"/>
-    <mergeCell ref="P22:R22"/>
-    <mergeCell ref="S22:U22"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="G21:I21"/>
-    <mergeCell ref="J21:L21"/>
-    <mergeCell ref="M21:O21"/>
-    <mergeCell ref="P21:R21"/>
-    <mergeCell ref="P24:R24"/>
-    <mergeCell ref="S24:U24"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="J25:L25"/>
-    <mergeCell ref="M25:O25"/>
-    <mergeCell ref="P25:R25"/>
-    <mergeCell ref="S25:U25"/>
-    <mergeCell ref="S26:U26"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="D27:F27"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="J27:L27"/>
-    <mergeCell ref="M27:O27"/>
-    <mergeCell ref="P27:R27"/>
-    <mergeCell ref="S27:U27"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="D26:F26"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="J26:L26"/>
-    <mergeCell ref="M26:O26"/>
-    <mergeCell ref="P26:R26"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="D31:F31"/>
-    <mergeCell ref="G31:I31"/>
-    <mergeCell ref="J31:L31"/>
-    <mergeCell ref="M31:O31"/>
-    <mergeCell ref="S28:U28"/>
-    <mergeCell ref="D29:F29"/>
-    <mergeCell ref="G29:I29"/>
-    <mergeCell ref="J29:L29"/>
-    <mergeCell ref="M29:O29"/>
-    <mergeCell ref="P29:R29"/>
-    <mergeCell ref="S29:U29"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="D28:F28"/>
-    <mergeCell ref="G28:I28"/>
-    <mergeCell ref="J28:L28"/>
-    <mergeCell ref="M28:O28"/>
-    <mergeCell ref="P28:R28"/>
-    <mergeCell ref="P31:R31"/>
-    <mergeCell ref="S31:U31"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="D32:F32"/>
-    <mergeCell ref="G32:I32"/>
-    <mergeCell ref="J32:L32"/>
-    <mergeCell ref="M32:O32"/>
-    <mergeCell ref="P32:R32"/>
-    <mergeCell ref="S32:U32"/>
-    <mergeCell ref="S33:U33"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="D34:F34"/>
-    <mergeCell ref="G34:I34"/>
-    <mergeCell ref="J34:L34"/>
-    <mergeCell ref="M34:O34"/>
-    <mergeCell ref="P34:R34"/>
-    <mergeCell ref="S34:U34"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="D33:F33"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="J33:L33"/>
-    <mergeCell ref="M33:O33"/>
-    <mergeCell ref="P33:R33"/>
-    <mergeCell ref="Q54:U54"/>
-    <mergeCell ref="A43:U46"/>
-    <mergeCell ref="A49:D49"/>
-    <mergeCell ref="J49:M49"/>
-    <mergeCell ref="R49:U49"/>
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="J53:M53"/>
-    <mergeCell ref="R53:U53"/>
-    <mergeCell ref="S35:U35"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="D36:F36"/>
-    <mergeCell ref="G36:I36"/>
-    <mergeCell ref="J36:L36"/>
-    <mergeCell ref="M36:O36"/>
-    <mergeCell ref="P36:R36"/>
-    <mergeCell ref="S36:U36"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="D35:F35"/>
-    <mergeCell ref="G35:I35"/>
-    <mergeCell ref="J35:L35"/>
-    <mergeCell ref="M35:O35"/>
-    <mergeCell ref="P35:R35"/>
-    <mergeCell ref="J50:M52"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
feat: Adjust battery export layout for improved data presentation
</commit_message>
<xml_diff>
--- a/public/assets/templates/maintenance/battery.xlsx
+++ b/public/assets/templates/maintenance/battery.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\maintenance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{420230AB-56C6-42FC-B5FF-70051445344B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26EE4FD6-4C6F-4E3C-A6A4-21A9051DD325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{632ED090-5FEF-4C64-87E3-52D42BEDE752}"/>
   </bookViews>
@@ -500,6 +500,72 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -512,15 +578,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -529,63 +586,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -968,54 +968,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="15" thickTop="1">
-      <c r="A1" s="34"/>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="37" t="s">
+      <c r="A1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-      <c r="K1" s="38"/>
-      <c r="L1" s="38"/>
-      <c r="M1" s="38"/>
-      <c r="N1" s="38"/>
-      <c r="O1" s="38"/>
-      <c r="P1" s="38"/>
-      <c r="Q1" s="38"/>
-      <c r="R1" s="38"/>
-      <c r="S1" s="38"/>
-      <c r="T1" s="38"/>
-      <c r="U1" s="39"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
+      <c r="S1" s="29"/>
+      <c r="T1" s="29"/>
+      <c r="U1" s="30"/>
     </row>
     <row r="2" spans="1:21">
-      <c r="A2" s="36"/>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="40" t="s">
+      <c r="A2" s="26"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41"/>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41"/>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="41"/>
-      <c r="Q2" s="41"/>
-      <c r="R2" s="41"/>
-      <c r="S2" s="41"/>
-      <c r="T2" s="41"/>
-      <c r="U2" s="42"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="32"/>
+      <c r="Q2" s="32"/>
+      <c r="R2" s="32"/>
+      <c r="S2" s="32"/>
+      <c r="T2" s="32"/>
+      <c r="U2" s="33"/>
     </row>
     <row r="3" spans="1:21">
       <c r="A3" s="1"/>
@@ -1023,14 +1023,14 @@
       <c r="U3" s="3"/>
     </row>
     <row r="4" spans="1:21">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="43"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="43"/>
-      <c r="F4" s="43"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
       <c r="G4" s="4"/>
       <c r="H4" t="s">
         <v>3</v>
@@ -1058,14 +1058,14 @@
       <c r="U5" s="3"/>
     </row>
     <row r="6" spans="1:21">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="43"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="43"/>
-      <c r="F6" s="43"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="35"/>
+      <c r="F6" s="35"/>
       <c r="G6" s="7"/>
       <c r="H6" t="s">
         <v>6</v>
@@ -1093,11 +1093,11 @@
       <c r="U8" s="3"/>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="30" t="s">
+      <c r="A9" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="31"/>
-      <c r="C9" s="31"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
       <c r="D9" s="9" t="s">
         <v>8</v>
       </c>
@@ -1154,61 +1154,61 @@
       </c>
     </row>
     <row r="10" spans="1:21">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="29"/>
-      <c r="C10" s="29"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="32"/>
-      <c r="H10" s="32"/>
-      <c r="I10" s="32"/>
-      <c r="J10" s="32"/>
-      <c r="K10" s="32"/>
-      <c r="L10" s="32"/>
-      <c r="M10" s="32"/>
-      <c r="N10" s="32"/>
-      <c r="O10" s="32"/>
-      <c r="P10" s="32"/>
-      <c r="Q10" s="32"/>
-      <c r="R10" s="32"/>
-      <c r="S10" s="32"/>
-      <c r="T10" s="32"/>
-      <c r="U10" s="33"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="23"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
+      <c r="M10" s="23"/>
+      <c r="N10" s="23"/>
+      <c r="O10" s="23"/>
+      <c r="P10" s="23"/>
+      <c r="Q10" s="23"/>
+      <c r="R10" s="23"/>
+      <c r="S10" s="23"/>
+      <c r="T10" s="23"/>
+      <c r="U10" s="36"/>
     </row>
     <row r="11" spans="1:21">
-      <c r="A11" s="28" t="s">
+      <c r="A11" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="29"/>
-      <c r="C11" s="29"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
-      <c r="J11" s="26"/>
-      <c r="K11" s="26"/>
-      <c r="L11" s="26"/>
-      <c r="M11" s="26"/>
-      <c r="N11" s="26"/>
-      <c r="O11" s="26"/>
-      <c r="P11" s="26"/>
-      <c r="Q11" s="26"/>
-      <c r="R11" s="26"/>
-      <c r="S11" s="26"/>
-      <c r="T11" s="26"/>
-      <c r="U11" s="27"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="27"/>
+      <c r="K11" s="27"/>
+      <c r="L11" s="27"/>
+      <c r="M11" s="27"/>
+      <c r="N11" s="27"/>
+      <c r="O11" s="27"/>
+      <c r="P11" s="27"/>
+      <c r="Q11" s="27"/>
+      <c r="R11" s="27"/>
+      <c r="S11" s="27"/>
+      <c r="T11" s="27"/>
+      <c r="U11" s="37"/>
     </row>
     <row r="12" spans="1:21">
-      <c r="A12" s="30" t="s">
+      <c r="A12" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="31"/>
-      <c r="C12" s="31"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
       <c r="D12" s="12" t="s">
         <v>8</v>
       </c>
@@ -1265,61 +1265,61 @@
       </c>
     </row>
     <row r="13" spans="1:21">
-      <c r="A13" s="28" t="s">
+      <c r="A13" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="29"/>
-      <c r="C13" s="29"/>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="32"/>
-      <c r="H13" s="32"/>
-      <c r="I13" s="32"/>
-      <c r="J13" s="32"/>
-      <c r="K13" s="32"/>
-      <c r="L13" s="32"/>
-      <c r="M13" s="32"/>
-      <c r="N13" s="32"/>
-      <c r="O13" s="32"/>
-      <c r="P13" s="32"/>
-      <c r="Q13" s="32"/>
-      <c r="R13" s="32"/>
-      <c r="S13" s="32"/>
-      <c r="T13" s="32"/>
-      <c r="U13" s="33"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="23"/>
+      <c r="I13" s="23"/>
+      <c r="J13" s="23"/>
+      <c r="K13" s="23"/>
+      <c r="L13" s="23"/>
+      <c r="M13" s="23"/>
+      <c r="N13" s="23"/>
+      <c r="O13" s="23"/>
+      <c r="P13" s="23"/>
+      <c r="Q13" s="23"/>
+      <c r="R13" s="23"/>
+      <c r="S13" s="23"/>
+      <c r="T13" s="23"/>
+      <c r="U13" s="36"/>
     </row>
     <row r="14" spans="1:21">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="29"/>
-      <c r="C14" s="29"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="26"/>
-      <c r="J14" s="26"/>
-      <c r="K14" s="26"/>
-      <c r="L14" s="26"/>
-      <c r="M14" s="26"/>
-      <c r="N14" s="26"/>
-      <c r="O14" s="26"/>
-      <c r="P14" s="26"/>
-      <c r="Q14" s="26"/>
-      <c r="R14" s="26"/>
-      <c r="S14" s="26"/>
-      <c r="T14" s="26"/>
-      <c r="U14" s="27"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="27"/>
+      <c r="K14" s="27"/>
+      <c r="L14" s="27"/>
+      <c r="M14" s="27"/>
+      <c r="N14" s="27"/>
+      <c r="O14" s="27"/>
+      <c r="P14" s="27"/>
+      <c r="Q14" s="27"/>
+      <c r="R14" s="27"/>
+      <c r="S14" s="27"/>
+      <c r="T14" s="27"/>
+      <c r="U14" s="37"/>
     </row>
     <row r="15" spans="1:21">
-      <c r="A15" s="30" t="s">
+      <c r="A15" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="31"/>
-      <c r="C15" s="31"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
       <c r="D15" s="12" t="s">
         <v>8</v>
       </c>
@@ -1376,61 +1376,61 @@
       </c>
     </row>
     <row r="16" spans="1:21">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="29"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="32"/>
-      <c r="H16" s="32"/>
-      <c r="I16" s="32"/>
-      <c r="J16" s="32"/>
-      <c r="K16" s="32"/>
-      <c r="L16" s="32"/>
-      <c r="M16" s="32"/>
-      <c r="N16" s="32"/>
-      <c r="O16" s="32"/>
-      <c r="P16" s="32"/>
-      <c r="Q16" s="32"/>
-      <c r="R16" s="32"/>
-      <c r="S16" s="32"/>
-      <c r="T16" s="32"/>
-      <c r="U16" s="33"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="23"/>
+      <c r="M16" s="23"/>
+      <c r="N16" s="23"/>
+      <c r="O16" s="23"/>
+      <c r="P16" s="23"/>
+      <c r="Q16" s="23"/>
+      <c r="R16" s="23"/>
+      <c r="S16" s="23"/>
+      <c r="T16" s="23"/>
+      <c r="U16" s="36"/>
     </row>
     <row r="17" spans="1:21">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="29"/>
-      <c r="C17" s="29"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="26"/>
-      <c r="H17" s="26"/>
-      <c r="I17" s="26"/>
-      <c r="J17" s="26"/>
-      <c r="K17" s="26"/>
-      <c r="L17" s="26"/>
-      <c r="M17" s="26"/>
-      <c r="N17" s="26"/>
-      <c r="O17" s="26"/>
-      <c r="P17" s="26"/>
-      <c r="Q17" s="26"/>
-      <c r="R17" s="26"/>
-      <c r="S17" s="26"/>
-      <c r="T17" s="26"/>
-      <c r="U17" s="27"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="27"/>
+      <c r="J17" s="27"/>
+      <c r="K17" s="27"/>
+      <c r="L17" s="27"/>
+      <c r="M17" s="27"/>
+      <c r="N17" s="27"/>
+      <c r="O17" s="27"/>
+      <c r="P17" s="27"/>
+      <c r="Q17" s="27"/>
+      <c r="R17" s="27"/>
+      <c r="S17" s="27"/>
+      <c r="T17" s="27"/>
+      <c r="U17" s="37"/>
     </row>
     <row r="18" spans="1:21">
-      <c r="A18" s="30" t="s">
+      <c r="A18" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="31"/>
-      <c r="C18" s="31"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
       <c r="D18" s="12" t="s">
         <v>8</v>
       </c>
@@ -1487,54 +1487,54 @@
       </c>
     </row>
     <row r="19" spans="1:21">
-      <c r="A19" s="28" t="s">
+      <c r="A19" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B19" s="29"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="32"/>
-      <c r="E19" s="32"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32"/>
-      <c r="H19" s="32"/>
-      <c r="I19" s="32"/>
-      <c r="J19" s="32"/>
-      <c r="K19" s="32"/>
-      <c r="L19" s="32"/>
-      <c r="M19" s="32"/>
-      <c r="N19" s="32"/>
-      <c r="O19" s="32"/>
-      <c r="P19" s="32"/>
-      <c r="Q19" s="32"/>
-      <c r="R19" s="32"/>
-      <c r="S19" s="32"/>
-      <c r="T19" s="32"/>
-      <c r="U19" s="33"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
+      <c r="G19" s="23"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
+      <c r="J19" s="23"/>
+      <c r="K19" s="23"/>
+      <c r="L19" s="23"/>
+      <c r="M19" s="23"/>
+      <c r="N19" s="23"/>
+      <c r="O19" s="23"/>
+      <c r="P19" s="23"/>
+      <c r="Q19" s="23"/>
+      <c r="R19" s="23"/>
+      <c r="S19" s="23"/>
+      <c r="T19" s="23"/>
+      <c r="U19" s="36"/>
     </row>
     <row r="20" spans="1:21">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="29"/>
-      <c r="C20" s="29"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
-      <c r="I20" s="26"/>
-      <c r="J20" s="26"/>
-      <c r="K20" s="26"/>
-      <c r="L20" s="26"/>
-      <c r="M20" s="26"/>
-      <c r="N20" s="26"/>
-      <c r="O20" s="26"/>
-      <c r="P20" s="26"/>
-      <c r="Q20" s="26"/>
-      <c r="R20" s="26"/>
-      <c r="S20" s="26"/>
-      <c r="T20" s="26"/>
-      <c r="U20" s="27"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="27"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="27"/>
+      <c r="K20" s="27"/>
+      <c r="L20" s="27"/>
+      <c r="M20" s="27"/>
+      <c r="N20" s="27"/>
+      <c r="O20" s="27"/>
+      <c r="P20" s="27"/>
+      <c r="Q20" s="27"/>
+      <c r="R20" s="27"/>
+      <c r="S20" s="27"/>
+      <c r="T20" s="27"/>
+      <c r="U20" s="37"/>
     </row>
     <row r="21" spans="1:21">
       <c r="A21" s="1"/>
@@ -1593,11 +1593,11 @@
       <c r="N25" t="s">
         <v>31</v>
       </c>
-      <c r="R25" s="44" t="s">
+      <c r="R25" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="S25" s="44"/>
-      <c r="T25" s="44"/>
+      <c r="S25" s="16"/>
+      <c r="T25" s="16"/>
       <c r="U25" s="3"/>
     </row>
     <row r="26" spans="1:21">
@@ -1605,11 +1605,11 @@
       <c r="N26" t="s">
         <v>32</v>
       </c>
-      <c r="R26" s="44" t="s">
+      <c r="R26" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="S26" s="44"/>
-      <c r="T26" s="44"/>
+      <c r="S26" s="16"/>
+      <c r="T26" s="16"/>
       <c r="U26" s="3"/>
     </row>
     <row r="27" spans="1:21">
@@ -1617,11 +1617,11 @@
       <c r="N27" t="s">
         <v>33</v>
       </c>
-      <c r="R27" s="44" t="s">
+      <c r="R27" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="S27" s="44"/>
-      <c r="T27" s="44"/>
+      <c r="S27" s="16"/>
+      <c r="T27" s="16"/>
       <c r="U27" s="3"/>
     </row>
     <row r="28" spans="1:21">
@@ -1629,11 +1629,11 @@
       <c r="N28" t="s">
         <v>34</v>
       </c>
-      <c r="R28" s="44" t="s">
+      <c r="R28" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="S28" s="44"/>
-      <c r="T28" s="44"/>
+      <c r="S28" s="16"/>
+      <c r="T28" s="16"/>
       <c r="U28" s="3"/>
     </row>
     <row r="29" spans="1:21">
@@ -1641,98 +1641,98 @@
       <c r="U29" s="3"/>
     </row>
     <row r="30" spans="1:21">
-      <c r="A30" s="17" t="s">
+      <c r="A30" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="B30" s="18"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
-      <c r="F30" s="18"/>
-      <c r="G30" s="18"/>
-      <c r="H30" s="18"/>
-      <c r="I30" s="18"/>
-      <c r="J30" s="18"/>
-      <c r="K30" s="18"/>
-      <c r="L30" s="18"/>
-      <c r="M30" s="18"/>
-      <c r="N30" s="18"/>
-      <c r="O30" s="18"/>
-      <c r="P30" s="18"/>
-      <c r="Q30" s="18"/>
-      <c r="R30" s="18"/>
-      <c r="S30" s="18"/>
-      <c r="T30" s="18"/>
-      <c r="U30" s="19"/>
+      <c r="B30" s="40"/>
+      <c r="C30" s="40"/>
+      <c r="D30" s="40"/>
+      <c r="E30" s="40"/>
+      <c r="F30" s="40"/>
+      <c r="G30" s="40"/>
+      <c r="H30" s="40"/>
+      <c r="I30" s="40"/>
+      <c r="J30" s="40"/>
+      <c r="K30" s="40"/>
+      <c r="L30" s="40"/>
+      <c r="M30" s="40"/>
+      <c r="N30" s="40"/>
+      <c r="O30" s="40"/>
+      <c r="P30" s="40"/>
+      <c r="Q30" s="40"/>
+      <c r="R30" s="40"/>
+      <c r="S30" s="40"/>
+      <c r="T30" s="40"/>
+      <c r="U30" s="41"/>
     </row>
     <row r="31" spans="1:21">
-      <c r="A31" s="17"/>
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="18"/>
-      <c r="F31" s="18"/>
-      <c r="G31" s="18"/>
-      <c r="H31" s="18"/>
-      <c r="I31" s="18"/>
-      <c r="J31" s="18"/>
-      <c r="K31" s="18"/>
-      <c r="L31" s="18"/>
-      <c r="M31" s="18"/>
-      <c r="N31" s="18"/>
-      <c r="O31" s="18"/>
-      <c r="P31" s="18"/>
-      <c r="Q31" s="18"/>
-      <c r="R31" s="18"/>
-      <c r="S31" s="18"/>
-      <c r="T31" s="18"/>
-      <c r="U31" s="19"/>
+      <c r="A31" s="39"/>
+      <c r="B31" s="40"/>
+      <c r="C31" s="40"/>
+      <c r="D31" s="40"/>
+      <c r="E31" s="40"/>
+      <c r="F31" s="40"/>
+      <c r="G31" s="40"/>
+      <c r="H31" s="40"/>
+      <c r="I31" s="40"/>
+      <c r="J31" s="40"/>
+      <c r="K31" s="40"/>
+      <c r="L31" s="40"/>
+      <c r="M31" s="40"/>
+      <c r="N31" s="40"/>
+      <c r="O31" s="40"/>
+      <c r="P31" s="40"/>
+      <c r="Q31" s="40"/>
+      <c r="R31" s="40"/>
+      <c r="S31" s="40"/>
+      <c r="T31" s="40"/>
+      <c r="U31" s="41"/>
     </row>
     <row r="32" spans="1:21">
-      <c r="A32" s="17"/>
-      <c r="B32" s="18"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="18"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="18"/>
-      <c r="G32" s="18"/>
-      <c r="H32" s="18"/>
-      <c r="I32" s="18"/>
-      <c r="J32" s="18"/>
-      <c r="K32" s="18"/>
-      <c r="L32" s="18"/>
-      <c r="M32" s="18"/>
-      <c r="N32" s="18"/>
-      <c r="O32" s="18"/>
-      <c r="P32" s="18"/>
-      <c r="Q32" s="18"/>
-      <c r="R32" s="18"/>
-      <c r="S32" s="18"/>
-      <c r="T32" s="18"/>
-      <c r="U32" s="19"/>
+      <c r="A32" s="39"/>
+      <c r="B32" s="40"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="40"/>
+      <c r="E32" s="40"/>
+      <c r="F32" s="40"/>
+      <c r="G32" s="40"/>
+      <c r="H32" s="40"/>
+      <c r="I32" s="40"/>
+      <c r="J32" s="40"/>
+      <c r="K32" s="40"/>
+      <c r="L32" s="40"/>
+      <c r="M32" s="40"/>
+      <c r="N32" s="40"/>
+      <c r="O32" s="40"/>
+      <c r="P32" s="40"/>
+      <c r="Q32" s="40"/>
+      <c r="R32" s="40"/>
+      <c r="S32" s="40"/>
+      <c r="T32" s="40"/>
+      <c r="U32" s="41"/>
     </row>
     <row r="33" spans="1:21">
-      <c r="A33" s="17"/>
-      <c r="B33" s="18"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="18"/>
-      <c r="H33" s="18"/>
-      <c r="I33" s="18"/>
-      <c r="J33" s="18"/>
-      <c r="K33" s="18"/>
-      <c r="L33" s="18"/>
-      <c r="M33" s="18"/>
-      <c r="N33" s="18"/>
-      <c r="O33" s="18"/>
-      <c r="P33" s="18"/>
-      <c r="Q33" s="18"/>
-      <c r="R33" s="18"/>
-      <c r="S33" s="18"/>
-      <c r="T33" s="18"/>
-      <c r="U33" s="19"/>
+      <c r="A33" s="39"/>
+      <c r="B33" s="40"/>
+      <c r="C33" s="40"/>
+      <c r="D33" s="40"/>
+      <c r="E33" s="40"/>
+      <c r="F33" s="40"/>
+      <c r="G33" s="40"/>
+      <c r="H33" s="40"/>
+      <c r="I33" s="40"/>
+      <c r="J33" s="40"/>
+      <c r="K33" s="40"/>
+      <c r="L33" s="40"/>
+      <c r="M33" s="40"/>
+      <c r="N33" s="40"/>
+      <c r="O33" s="40"/>
+      <c r="P33" s="40"/>
+      <c r="Q33" s="40"/>
+      <c r="R33" s="40"/>
+      <c r="S33" s="40"/>
+      <c r="T33" s="40"/>
+      <c r="U33" s="41"/>
     </row>
     <row r="34" spans="1:21">
       <c r="A34" s="1"/>
@@ -1743,173 +1743,107 @@
       <c r="U35" s="3"/>
     </row>
     <row r="36" spans="1:21">
-      <c r="A36" s="20" t="s">
+      <c r="A36" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="B36" s="21"/>
-      <c r="C36" s="21"/>
-      <c r="D36" s="21"/>
-      <c r="J36" s="21" t="s">
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="J36" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K36" s="21"/>
-      <c r="L36" s="21"/>
-      <c r="M36" s="21"/>
-      <c r="R36" s="21" t="s">
+      <c r="K36" s="17"/>
+      <c r="L36" s="17"/>
+      <c r="M36" s="17"/>
+      <c r="R36" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="S36" s="21"/>
-      <c r="T36" s="21"/>
-      <c r="U36" s="22"/>
+      <c r="S36" s="17"/>
+      <c r="T36" s="17"/>
+      <c r="U36" s="18"/>
     </row>
     <row r="37" spans="1:21">
-      <c r="A37" s="20"/>
-      <c r="B37" s="21"/>
-      <c r="C37" s="21"/>
-      <c r="D37" s="21"/>
-      <c r="J37" s="21"/>
-      <c r="K37" s="21"/>
-      <c r="L37" s="21"/>
-      <c r="M37" s="21"/>
-      <c r="R37" s="21"/>
-      <c r="S37" s="21"/>
-      <c r="T37" s="21"/>
-      <c r="U37" s="22"/>
+      <c r="A37" s="34"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="J37" s="17"/>
+      <c r="K37" s="17"/>
+      <c r="L37" s="17"/>
+      <c r="M37" s="17"/>
+      <c r="R37" s="17"/>
+      <c r="S37" s="17"/>
+      <c r="T37" s="17"/>
+      <c r="U37" s="18"/>
     </row>
     <row r="38" spans="1:21">
-      <c r="A38" s="20"/>
-      <c r="B38" s="21"/>
-      <c r="C38" s="21"/>
-      <c r="D38" s="21"/>
-      <c r="J38" s="21"/>
-      <c r="K38" s="21"/>
-      <c r="L38" s="21"/>
-      <c r="M38" s="21"/>
-      <c r="R38" s="21"/>
-      <c r="S38" s="21"/>
-      <c r="T38" s="21"/>
-      <c r="U38" s="22"/>
+      <c r="A38" s="34"/>
+      <c r="B38" s="17"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="J38" s="17"/>
+      <c r="K38" s="17"/>
+      <c r="L38" s="17"/>
+      <c r="M38" s="17"/>
+      <c r="R38" s="17"/>
+      <c r="S38" s="17"/>
+      <c r="T38" s="17"/>
+      <c r="U38" s="18"/>
     </row>
     <row r="39" spans="1:21">
-      <c r="A39" s="20"/>
-      <c r="B39" s="21"/>
-      <c r="C39" s="21"/>
-      <c r="D39" s="21"/>
-      <c r="J39" s="21"/>
-      <c r="K39" s="21"/>
-      <c r="L39" s="21"/>
-      <c r="M39" s="21"/>
-      <c r="R39" s="21"/>
-      <c r="S39" s="21"/>
-      <c r="T39" s="21"/>
-      <c r="U39" s="22"/>
+      <c r="A39" s="34"/>
+      <c r="B39" s="17"/>
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="J39" s="17"/>
+      <c r="K39" s="17"/>
+      <c r="L39" s="17"/>
+      <c r="M39" s="17"/>
+      <c r="R39" s="17"/>
+      <c r="S39" s="17"/>
+      <c r="T39" s="17"/>
+      <c r="U39" s="18"/>
     </row>
     <row r="40" spans="1:21" ht="15" thickBot="1">
-      <c r="A40" s="23" t="s">
+      <c r="A40" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="B40" s="24"/>
-      <c r="C40" s="24"/>
-      <c r="D40" s="24"/>
+      <c r="B40" s="43"/>
+      <c r="C40" s="43"/>
+      <c r="D40" s="43"/>
       <c r="E40" s="15"/>
       <c r="F40" s="15"/>
       <c r="G40" s="15"/>
       <c r="H40" s="15"/>
       <c r="I40" s="15"/>
-      <c r="J40" s="24" t="s">
+      <c r="J40" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="K40" s="24"/>
-      <c r="L40" s="24"/>
-      <c r="M40" s="24"/>
+      <c r="K40" s="43"/>
+      <c r="L40" s="43"/>
+      <c r="M40" s="43"/>
       <c r="N40" s="15"/>
       <c r="O40" s="15"/>
       <c r="P40" s="15"/>
       <c r="Q40" s="15"/>
-      <c r="R40" s="24" t="s">
+      <c r="R40" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="S40" s="24"/>
-      <c r="T40" s="24"/>
-      <c r="U40" s="25"/>
+      <c r="S40" s="43"/>
+      <c r="T40" s="43"/>
+      <c r="U40" s="44"/>
     </row>
     <row r="41" spans="1:21" ht="15" thickTop="1">
-      <c r="Q41" s="16" t="s">
+      <c r="Q41" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="R41" s="16"/>
-      <c r="S41" s="16"/>
-      <c r="T41" s="16"/>
-      <c r="U41" s="16"/>
+      <c r="R41" s="38"/>
+      <c r="S41" s="38"/>
+      <c r="T41" s="38"/>
+      <c r="U41" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="78">
-    <mergeCell ref="R37:U39"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="M10:O10"/>
-    <mergeCell ref="A1:D2"/>
-    <mergeCell ref="E1:U1"/>
-    <mergeCell ref="E2:U2"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="P10:R10"/>
-    <mergeCell ref="S10:U10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="P11:R11"/>
-    <mergeCell ref="S11:U11"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="M13:O13"/>
-    <mergeCell ref="P13:R13"/>
-    <mergeCell ref="S13:U13"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="M14:O14"/>
-    <mergeCell ref="P14:R14"/>
-    <mergeCell ref="S14:U14"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="J16:L16"/>
-    <mergeCell ref="M16:O16"/>
-    <mergeCell ref="P16:R16"/>
-    <mergeCell ref="S16:U16"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="M17:O17"/>
-    <mergeCell ref="P17:R17"/>
-    <mergeCell ref="S17:U17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="P19:R19"/>
-    <mergeCell ref="S19:U19"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="J20:L20"/>
-    <mergeCell ref="M20:O20"/>
     <mergeCell ref="P20:R20"/>
     <mergeCell ref="S20:U20"/>
     <mergeCell ref="Q41:U41"/>
@@ -1922,6 +1856,72 @@
     <mergeCell ref="R40:U40"/>
     <mergeCell ref="J37:M39"/>
     <mergeCell ref="A37:D39"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="M20:O20"/>
+    <mergeCell ref="P17:R17"/>
+    <mergeCell ref="S17:U17"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="P19:R19"/>
+    <mergeCell ref="S19:U19"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="M17:O17"/>
+    <mergeCell ref="S14:U14"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="J16:L16"/>
+    <mergeCell ref="M16:O16"/>
+    <mergeCell ref="P16:R16"/>
+    <mergeCell ref="S16:U16"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="M14:O14"/>
+    <mergeCell ref="P14:R14"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="P10:R10"/>
+    <mergeCell ref="S10:U10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="P11:R11"/>
+    <mergeCell ref="S11:U11"/>
+    <mergeCell ref="A1:D2"/>
+    <mergeCell ref="E1:U1"/>
+    <mergeCell ref="E2:U2"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="R37:U39"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="M10:O10"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="M13:O13"/>
+    <mergeCell ref="P13:R13"/>
+    <mergeCell ref="S13:U13"/>
+    <mergeCell ref="A14:C14"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
feat: merge cell for header information
</commit_message>
<xml_diff>
--- a/public/assets/templates/maintenance/battery.xlsx
+++ b/public/assets/templates/maintenance/battery.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\maintenance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26EE4FD6-4C6F-4E3C-A6A4-21A9051DD325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA4143BF-B41D-411B-A1D3-033153053317}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{632ED090-5FEF-4C64-87E3-52D42BEDE752}"/>
   </bookViews>
@@ -136,7 +136,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -176,6 +176,12 @@
       <name val="Arial"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -451,7 +457,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -503,16 +509,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -521,9 +551,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -533,9 +572,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -554,38 +590,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -968,54 +980,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="15" thickTop="1">
-      <c r="A1" s="24"/>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="28" t="s">
+      <c r="A1" s="35"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="29"/>
-      <c r="O1" s="29"/>
-      <c r="P1" s="29"/>
-      <c r="Q1" s="29"/>
-      <c r="R1" s="29"/>
-      <c r="S1" s="29"/>
-      <c r="T1" s="29"/>
-      <c r="U1" s="30"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="39"/>
+      <c r="P1" s="39"/>
+      <c r="Q1" s="39"/>
+      <c r="R1" s="39"/>
+      <c r="S1" s="39"/>
+      <c r="T1" s="39"/>
+      <c r="U1" s="40"/>
     </row>
     <row r="2" spans="1:21">
-      <c r="A2" s="26"/>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="31" t="s">
+      <c r="A2" s="37"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="32"/>
-      <c r="P2" s="32"/>
-      <c r="Q2" s="32"/>
-      <c r="R2" s="32"/>
-      <c r="S2" s="32"/>
-      <c r="T2" s="32"/>
-      <c r="U2" s="33"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42"/>
+      <c r="O2" s="42"/>
+      <c r="P2" s="42"/>
+      <c r="Q2" s="42"/>
+      <c r="R2" s="42"/>
+      <c r="S2" s="42"/>
+      <c r="T2" s="42"/>
+      <c r="U2" s="43"/>
     </row>
     <row r="3" spans="1:21">
       <c r="A3" s="1"/>
@@ -1023,28 +1035,28 @@
       <c r="U3" s="3"/>
     </row>
     <row r="4" spans="1:21">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="35"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="44"/>
+      <c r="F4" s="44"/>
       <c r="G4" s="4"/>
       <c r="H4" t="s">
         <v>3</v>
       </c>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
+      <c r="K4" s="45"/>
+      <c r="L4" s="45"/>
+      <c r="M4" s="45"/>
+      <c r="N4" s="45"/>
       <c r="P4" t="s">
         <v>4</v>
       </c>
-      <c r="R4" s="5"/>
-      <c r="S4" s="5"/>
-      <c r="T4" s="5"/>
+      <c r="R4" s="45"/>
+      <c r="S4" s="45"/>
+      <c r="T4" s="45"/>
       <c r="U4" s="3"/>
     </row>
     <row r="5" spans="1:21">
@@ -1058,22 +1070,22 @@
       <c r="U5" s="3"/>
     </row>
     <row r="6" spans="1:21">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="35"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="35"/>
-      <c r="F6" s="35"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
       <c r="G6" s="7"/>
       <c r="H6" t="s">
         <v>6</v>
       </c>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
+      <c r="K6" s="46"/>
+      <c r="L6" s="46"/>
+      <c r="M6" s="46"/>
+      <c r="N6" s="46"/>
       <c r="U6" s="3"/>
     </row>
     <row r="7" spans="1:21">
@@ -1093,11 +1105,11 @@
       <c r="U8" s="3"/>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
+      <c r="B9" s="32"/>
+      <c r="C9" s="32"/>
       <c r="D9" s="9" t="s">
         <v>8</v>
       </c>
@@ -1154,61 +1166,61 @@
       </c>
     </row>
     <row r="10" spans="1:21">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="23"/>
-      <c r="M10" s="23"/>
-      <c r="N10" s="23"/>
-      <c r="O10" s="23"/>
-      <c r="P10" s="23"/>
-      <c r="Q10" s="23"/>
-      <c r="R10" s="23"/>
-      <c r="S10" s="23"/>
-      <c r="T10" s="23"/>
-      <c r="U10" s="36"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="33"/>
+      <c r="J10" s="33"/>
+      <c r="K10" s="33"/>
+      <c r="L10" s="33"/>
+      <c r="M10" s="33"/>
+      <c r="N10" s="33"/>
+      <c r="O10" s="33"/>
+      <c r="P10" s="33"/>
+      <c r="Q10" s="33"/>
+      <c r="R10" s="33"/>
+      <c r="S10" s="33"/>
+      <c r="T10" s="33"/>
+      <c r="U10" s="34"/>
     </row>
     <row r="11" spans="1:21">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="22"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="27"/>
-      <c r="J11" s="27"/>
-      <c r="K11" s="27"/>
-      <c r="L11" s="27"/>
-      <c r="M11" s="27"/>
-      <c r="N11" s="27"/>
-      <c r="O11" s="27"/>
-      <c r="P11" s="27"/>
-      <c r="Q11" s="27"/>
-      <c r="R11" s="27"/>
-      <c r="S11" s="27"/>
-      <c r="T11" s="27"/>
-      <c r="U11" s="37"/>
+      <c r="B11" s="30"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="17"/>
+      <c r="L11" s="17"/>
+      <c r="M11" s="17"/>
+      <c r="N11" s="17"/>
+      <c r="O11" s="17"/>
+      <c r="P11" s="17"/>
+      <c r="Q11" s="17"/>
+      <c r="R11" s="17"/>
+      <c r="S11" s="17"/>
+      <c r="T11" s="17"/>
+      <c r="U11" s="18"/>
     </row>
     <row r="12" spans="1:21">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
+      <c r="B12" s="32"/>
+      <c r="C12" s="32"/>
       <c r="D12" s="12" t="s">
         <v>8</v>
       </c>
@@ -1265,61 +1277,61 @@
       </c>
     </row>
     <row r="13" spans="1:21">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="22"/>
-      <c r="C13" s="22"/>
-      <c r="D13" s="23"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="23"/>
-      <c r="I13" s="23"/>
-      <c r="J13" s="23"/>
-      <c r="K13" s="23"/>
-      <c r="L13" s="23"/>
-      <c r="M13" s="23"/>
-      <c r="N13" s="23"/>
-      <c r="O13" s="23"/>
-      <c r="P13" s="23"/>
-      <c r="Q13" s="23"/>
-      <c r="R13" s="23"/>
-      <c r="S13" s="23"/>
-      <c r="T13" s="23"/>
-      <c r="U13" s="36"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="33"/>
+      <c r="E13" s="33"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="33"/>
+      <c r="H13" s="33"/>
+      <c r="I13" s="33"/>
+      <c r="J13" s="33"/>
+      <c r="K13" s="33"/>
+      <c r="L13" s="33"/>
+      <c r="M13" s="33"/>
+      <c r="N13" s="33"/>
+      <c r="O13" s="33"/>
+      <c r="P13" s="33"/>
+      <c r="Q13" s="33"/>
+      <c r="R13" s="33"/>
+      <c r="S13" s="33"/>
+      <c r="T13" s="33"/>
+      <c r="U13" s="34"/>
     </row>
     <row r="14" spans="1:21">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="22"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="27"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="27"/>
-      <c r="I14" s="27"/>
-      <c r="J14" s="27"/>
-      <c r="K14" s="27"/>
-      <c r="L14" s="27"/>
-      <c r="M14" s="27"/>
-      <c r="N14" s="27"/>
-      <c r="O14" s="27"/>
-      <c r="P14" s="27"/>
-      <c r="Q14" s="27"/>
-      <c r="R14" s="27"/>
-      <c r="S14" s="27"/>
-      <c r="T14" s="27"/>
-      <c r="U14" s="37"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="17"/>
+      <c r="M14" s="17"/>
+      <c r="N14" s="17"/>
+      <c r="O14" s="17"/>
+      <c r="P14" s="17"/>
+      <c r="Q14" s="17"/>
+      <c r="R14" s="17"/>
+      <c r="S14" s="17"/>
+      <c r="T14" s="17"/>
+      <c r="U14" s="18"/>
     </row>
     <row r="15" spans="1:21">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
+      <c r="B15" s="32"/>
+      <c r="C15" s="32"/>
       <c r="D15" s="12" t="s">
         <v>8</v>
       </c>
@@ -1376,61 +1388,61 @@
       </c>
     </row>
     <row r="16" spans="1:21">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="22"/>
-      <c r="C16" s="22"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="23"/>
-      <c r="M16" s="23"/>
-      <c r="N16" s="23"/>
-      <c r="O16" s="23"/>
-      <c r="P16" s="23"/>
-      <c r="Q16" s="23"/>
-      <c r="R16" s="23"/>
-      <c r="S16" s="23"/>
-      <c r="T16" s="23"/>
-      <c r="U16" s="36"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="33"/>
+      <c r="J16" s="33"/>
+      <c r="K16" s="33"/>
+      <c r="L16" s="33"/>
+      <c r="M16" s="33"/>
+      <c r="N16" s="33"/>
+      <c r="O16" s="33"/>
+      <c r="P16" s="33"/>
+      <c r="Q16" s="33"/>
+      <c r="R16" s="33"/>
+      <c r="S16" s="33"/>
+      <c r="T16" s="33"/>
+      <c r="U16" s="34"/>
     </row>
     <row r="17" spans="1:21">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="27"/>
-      <c r="J17" s="27"/>
-      <c r="K17" s="27"/>
-      <c r="L17" s="27"/>
-      <c r="M17" s="27"/>
-      <c r="N17" s="27"/>
-      <c r="O17" s="27"/>
-      <c r="P17" s="27"/>
-      <c r="Q17" s="27"/>
-      <c r="R17" s="27"/>
-      <c r="S17" s="27"/>
-      <c r="T17" s="27"/>
-      <c r="U17" s="37"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="17"/>
+      <c r="L17" s="17"/>
+      <c r="M17" s="17"/>
+      <c r="N17" s="17"/>
+      <c r="O17" s="17"/>
+      <c r="P17" s="17"/>
+      <c r="Q17" s="17"/>
+      <c r="R17" s="17"/>
+      <c r="S17" s="17"/>
+      <c r="T17" s="17"/>
+      <c r="U17" s="18"/>
     </row>
     <row r="18" spans="1:21">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
+      <c r="B18" s="32"/>
+      <c r="C18" s="32"/>
       <c r="D18" s="12" t="s">
         <v>8</v>
       </c>
@@ -1487,54 +1499,54 @@
       </c>
     </row>
     <row r="19" spans="1:21">
-      <c r="A19" s="21" t="s">
+      <c r="A19" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="23"/>
-      <c r="I19" s="23"/>
-      <c r="J19" s="23"/>
-      <c r="K19" s="23"/>
-      <c r="L19" s="23"/>
-      <c r="M19" s="23"/>
-      <c r="N19" s="23"/>
-      <c r="O19" s="23"/>
-      <c r="P19" s="23"/>
-      <c r="Q19" s="23"/>
-      <c r="R19" s="23"/>
-      <c r="S19" s="23"/>
-      <c r="T19" s="23"/>
-      <c r="U19" s="36"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="33"/>
+      <c r="I19" s="33"/>
+      <c r="J19" s="33"/>
+      <c r="K19" s="33"/>
+      <c r="L19" s="33"/>
+      <c r="M19" s="33"/>
+      <c r="N19" s="33"/>
+      <c r="O19" s="33"/>
+      <c r="P19" s="33"/>
+      <c r="Q19" s="33"/>
+      <c r="R19" s="33"/>
+      <c r="S19" s="33"/>
+      <c r="T19" s="33"/>
+      <c r="U19" s="34"/>
     </row>
     <row r="20" spans="1:21">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="22"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="27"/>
-      <c r="I20" s="27"/>
-      <c r="J20" s="27"/>
-      <c r="K20" s="27"/>
-      <c r="L20" s="27"/>
-      <c r="M20" s="27"/>
-      <c r="N20" s="27"/>
-      <c r="O20" s="27"/>
-      <c r="P20" s="27"/>
-      <c r="Q20" s="27"/>
-      <c r="R20" s="27"/>
-      <c r="S20" s="27"/>
-      <c r="T20" s="27"/>
-      <c r="U20" s="37"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="17"/>
+      <c r="L20" s="17"/>
+      <c r="M20" s="17"/>
+      <c r="N20" s="17"/>
+      <c r="O20" s="17"/>
+      <c r="P20" s="17"/>
+      <c r="Q20" s="17"/>
+      <c r="R20" s="17"/>
+      <c r="S20" s="17"/>
+      <c r="T20" s="17"/>
+      <c r="U20" s="18"/>
     </row>
     <row r="21" spans="1:21">
       <c r="A21" s="1"/>
@@ -1641,98 +1653,98 @@
       <c r="U29" s="3"/>
     </row>
     <row r="30" spans="1:21">
-      <c r="A30" s="39" t="s">
+      <c r="A30" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="B30" s="40"/>
-      <c r="C30" s="40"/>
-      <c r="D30" s="40"/>
-      <c r="E30" s="40"/>
-      <c r="F30" s="40"/>
-      <c r="G30" s="40"/>
-      <c r="H30" s="40"/>
-      <c r="I30" s="40"/>
-      <c r="J30" s="40"/>
-      <c r="K30" s="40"/>
-      <c r="L30" s="40"/>
-      <c r="M30" s="40"/>
-      <c r="N30" s="40"/>
-      <c r="O30" s="40"/>
-      <c r="P30" s="40"/>
-      <c r="Q30" s="40"/>
-      <c r="R30" s="40"/>
-      <c r="S30" s="40"/>
-      <c r="T30" s="40"/>
-      <c r="U30" s="41"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+      <c r="I30" s="21"/>
+      <c r="J30" s="21"/>
+      <c r="K30" s="21"/>
+      <c r="L30" s="21"/>
+      <c r="M30" s="21"/>
+      <c r="N30" s="21"/>
+      <c r="O30" s="21"/>
+      <c r="P30" s="21"/>
+      <c r="Q30" s="21"/>
+      <c r="R30" s="21"/>
+      <c r="S30" s="21"/>
+      <c r="T30" s="21"/>
+      <c r="U30" s="22"/>
     </row>
     <row r="31" spans="1:21">
-      <c r="A31" s="39"/>
-      <c r="B31" s="40"/>
-      <c r="C31" s="40"/>
-      <c r="D31" s="40"/>
-      <c r="E31" s="40"/>
-      <c r="F31" s="40"/>
-      <c r="G31" s="40"/>
-      <c r="H31" s="40"/>
-      <c r="I31" s="40"/>
-      <c r="J31" s="40"/>
-      <c r="K31" s="40"/>
-      <c r="L31" s="40"/>
-      <c r="M31" s="40"/>
-      <c r="N31" s="40"/>
-      <c r="O31" s="40"/>
-      <c r="P31" s="40"/>
-      <c r="Q31" s="40"/>
-      <c r="R31" s="40"/>
-      <c r="S31" s="40"/>
-      <c r="T31" s="40"/>
-      <c r="U31" s="41"/>
+      <c r="A31" s="20"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="21"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="21"/>
+      <c r="H31" s="21"/>
+      <c r="I31" s="21"/>
+      <c r="J31" s="21"/>
+      <c r="K31" s="21"/>
+      <c r="L31" s="21"/>
+      <c r="M31" s="21"/>
+      <c r="N31" s="21"/>
+      <c r="O31" s="21"/>
+      <c r="P31" s="21"/>
+      <c r="Q31" s="21"/>
+      <c r="R31" s="21"/>
+      <c r="S31" s="21"/>
+      <c r="T31" s="21"/>
+      <c r="U31" s="22"/>
     </row>
     <row r="32" spans="1:21">
-      <c r="A32" s="39"/>
-      <c r="B32" s="40"/>
-      <c r="C32" s="40"/>
-      <c r="D32" s="40"/>
-      <c r="E32" s="40"/>
-      <c r="F32" s="40"/>
-      <c r="G32" s="40"/>
-      <c r="H32" s="40"/>
-      <c r="I32" s="40"/>
-      <c r="J32" s="40"/>
-      <c r="K32" s="40"/>
-      <c r="L32" s="40"/>
-      <c r="M32" s="40"/>
-      <c r="N32" s="40"/>
-      <c r="O32" s="40"/>
-      <c r="P32" s="40"/>
-      <c r="Q32" s="40"/>
-      <c r="R32" s="40"/>
-      <c r="S32" s="40"/>
-      <c r="T32" s="40"/>
-      <c r="U32" s="41"/>
+      <c r="A32" s="20"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="21"/>
+      <c r="D32" s="21"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
+      <c r="I32" s="21"/>
+      <c r="J32" s="21"/>
+      <c r="K32" s="21"/>
+      <c r="L32" s="21"/>
+      <c r="M32" s="21"/>
+      <c r="N32" s="21"/>
+      <c r="O32" s="21"/>
+      <c r="P32" s="21"/>
+      <c r="Q32" s="21"/>
+      <c r="R32" s="21"/>
+      <c r="S32" s="21"/>
+      <c r="T32" s="21"/>
+      <c r="U32" s="22"/>
     </row>
     <row r="33" spans="1:21">
-      <c r="A33" s="39"/>
-      <c r="B33" s="40"/>
-      <c r="C33" s="40"/>
-      <c r="D33" s="40"/>
-      <c r="E33" s="40"/>
-      <c r="F33" s="40"/>
-      <c r="G33" s="40"/>
-      <c r="H33" s="40"/>
-      <c r="I33" s="40"/>
-      <c r="J33" s="40"/>
-      <c r="K33" s="40"/>
-      <c r="L33" s="40"/>
-      <c r="M33" s="40"/>
-      <c r="N33" s="40"/>
-      <c r="O33" s="40"/>
-      <c r="P33" s="40"/>
-      <c r="Q33" s="40"/>
-      <c r="R33" s="40"/>
-      <c r="S33" s="40"/>
-      <c r="T33" s="40"/>
-      <c r="U33" s="41"/>
+      <c r="A33" s="20"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="21"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
+      <c r="I33" s="21"/>
+      <c r="J33" s="21"/>
+      <c r="K33" s="21"/>
+      <c r="L33" s="21"/>
+      <c r="M33" s="21"/>
+      <c r="N33" s="21"/>
+      <c r="O33" s="21"/>
+      <c r="P33" s="21"/>
+      <c r="Q33" s="21"/>
+      <c r="R33" s="21"/>
+      <c r="S33" s="21"/>
+      <c r="T33" s="21"/>
+      <c r="U33" s="22"/>
     </row>
     <row r="34" spans="1:21">
       <c r="A34" s="1"/>
@@ -1743,107 +1755,172 @@
       <c r="U35" s="3"/>
     </row>
     <row r="36" spans="1:21">
-      <c r="A36" s="34" t="s">
+      <c r="A36" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="J36" s="17" t="s">
+      <c r="B36" s="24"/>
+      <c r="C36" s="24"/>
+      <c r="D36" s="24"/>
+      <c r="J36" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="K36" s="17"/>
-      <c r="L36" s="17"/>
-      <c r="M36" s="17"/>
-      <c r="R36" s="17" t="s">
+      <c r="K36" s="24"/>
+      <c r="L36" s="24"/>
+      <c r="M36" s="24"/>
+      <c r="R36" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="S36" s="17"/>
-      <c r="T36" s="17"/>
-      <c r="U36" s="18"/>
+      <c r="S36" s="24"/>
+      <c r="T36" s="24"/>
+      <c r="U36" s="25"/>
     </row>
     <row r="37" spans="1:21">
-      <c r="A37" s="34"/>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="17"/>
-      <c r="J37" s="17"/>
-      <c r="K37" s="17"/>
-      <c r="L37" s="17"/>
-      <c r="M37" s="17"/>
-      <c r="R37" s="17"/>
-      <c r="S37" s="17"/>
-      <c r="T37" s="17"/>
-      <c r="U37" s="18"/>
+      <c r="A37" s="23"/>
+      <c r="B37" s="24"/>
+      <c r="C37" s="24"/>
+      <c r="D37" s="24"/>
+      <c r="J37" s="24"/>
+      <c r="K37" s="24"/>
+      <c r="L37" s="24"/>
+      <c r="M37" s="24"/>
+      <c r="R37" s="24"/>
+      <c r="S37" s="24"/>
+      <c r="T37" s="24"/>
+      <c r="U37" s="25"/>
     </row>
     <row r="38" spans="1:21">
-      <c r="A38" s="34"/>
-      <c r="B38" s="17"/>
-      <c r="C38" s="17"/>
-      <c r="D38" s="17"/>
-      <c r="J38" s="17"/>
-      <c r="K38" s="17"/>
-      <c r="L38" s="17"/>
-      <c r="M38" s="17"/>
-      <c r="R38" s="17"/>
-      <c r="S38" s="17"/>
-      <c r="T38" s="17"/>
-      <c r="U38" s="18"/>
+      <c r="A38" s="23"/>
+      <c r="B38" s="24"/>
+      <c r="C38" s="24"/>
+      <c r="D38" s="24"/>
+      <c r="J38" s="24"/>
+      <c r="K38" s="24"/>
+      <c r="L38" s="24"/>
+      <c r="M38" s="24"/>
+      <c r="R38" s="24"/>
+      <c r="S38" s="24"/>
+      <c r="T38" s="24"/>
+      <c r="U38" s="25"/>
     </row>
     <row r="39" spans="1:21">
-      <c r="A39" s="34"/>
-      <c r="B39" s="17"/>
-      <c r="C39" s="17"/>
-      <c r="D39" s="17"/>
-      <c r="J39" s="17"/>
-      <c r="K39" s="17"/>
-      <c r="L39" s="17"/>
-      <c r="M39" s="17"/>
-      <c r="R39" s="17"/>
-      <c r="S39" s="17"/>
-      <c r="T39" s="17"/>
-      <c r="U39" s="18"/>
+      <c r="A39" s="23"/>
+      <c r="B39" s="24"/>
+      <c r="C39" s="24"/>
+      <c r="D39" s="24"/>
+      <c r="J39" s="24"/>
+      <c r="K39" s="24"/>
+      <c r="L39" s="24"/>
+      <c r="M39" s="24"/>
+      <c r="R39" s="24"/>
+      <c r="S39" s="24"/>
+      <c r="T39" s="24"/>
+      <c r="U39" s="25"/>
     </row>
     <row r="40" spans="1:21" ht="15" thickBot="1">
-      <c r="A40" s="42" t="s">
+      <c r="A40" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="B40" s="43"/>
-      <c r="C40" s="43"/>
-      <c r="D40" s="43"/>
+      <c r="B40" s="27"/>
+      <c r="C40" s="27"/>
+      <c r="D40" s="27"/>
       <c r="E40" s="15"/>
       <c r="F40" s="15"/>
       <c r="G40" s="15"/>
       <c r="H40" s="15"/>
       <c r="I40" s="15"/>
-      <c r="J40" s="43" t="s">
+      <c r="J40" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="K40" s="43"/>
-      <c r="L40" s="43"/>
-      <c r="M40" s="43"/>
+      <c r="K40" s="27"/>
+      <c r="L40" s="27"/>
+      <c r="M40" s="27"/>
       <c r="N40" s="15"/>
       <c r="O40" s="15"/>
       <c r="P40" s="15"/>
       <c r="Q40" s="15"/>
-      <c r="R40" s="43" t="s">
+      <c r="R40" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="S40" s="43"/>
-      <c r="T40" s="43"/>
-      <c r="U40" s="44"/>
+      <c r="S40" s="27"/>
+      <c r="T40" s="27"/>
+      <c r="U40" s="28"/>
     </row>
     <row r="41" spans="1:21" ht="15" thickTop="1">
-      <c r="Q41" s="38" t="s">
+      <c r="Q41" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="R41" s="38"/>
-      <c r="S41" s="38"/>
-      <c r="T41" s="38"/>
-      <c r="U41" s="38"/>
+      <c r="R41" s="19"/>
+      <c r="S41" s="19"/>
+      <c r="T41" s="19"/>
+      <c r="U41" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="78">
+  <mergeCells count="81">
+    <mergeCell ref="R37:U39"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="M10:O10"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="M13:O13"/>
+    <mergeCell ref="P13:R13"/>
+    <mergeCell ref="S13:U13"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A1:D2"/>
+    <mergeCell ref="E1:U1"/>
+    <mergeCell ref="E2:U2"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="K4:N4"/>
+    <mergeCell ref="R4:T4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="P10:R10"/>
+    <mergeCell ref="S10:U10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="P11:R11"/>
+    <mergeCell ref="S11:U11"/>
+    <mergeCell ref="K6:N6"/>
+    <mergeCell ref="S14:U14"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="J16:L16"/>
+    <mergeCell ref="M16:O16"/>
+    <mergeCell ref="P16:R16"/>
+    <mergeCell ref="S16:U16"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="M14:O14"/>
+    <mergeCell ref="P14:R14"/>
+    <mergeCell ref="M20:O20"/>
+    <mergeCell ref="P17:R17"/>
+    <mergeCell ref="S17:U17"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="P19:R19"/>
+    <mergeCell ref="S19:U19"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="M17:O17"/>
     <mergeCell ref="P20:R20"/>
     <mergeCell ref="S20:U20"/>
     <mergeCell ref="Q41:U41"/>
@@ -1860,68 +1937,6 @@
     <mergeCell ref="D20:F20"/>
     <mergeCell ref="G20:I20"/>
     <mergeCell ref="J20:L20"/>
-    <mergeCell ref="M20:O20"/>
-    <mergeCell ref="P17:R17"/>
-    <mergeCell ref="S17:U17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="P19:R19"/>
-    <mergeCell ref="S19:U19"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="M17:O17"/>
-    <mergeCell ref="S14:U14"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="J16:L16"/>
-    <mergeCell ref="M16:O16"/>
-    <mergeCell ref="P16:R16"/>
-    <mergeCell ref="S16:U16"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="M14:O14"/>
-    <mergeCell ref="P14:R14"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="P10:R10"/>
-    <mergeCell ref="S10:U10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="P11:R11"/>
-    <mergeCell ref="S11:U11"/>
-    <mergeCell ref="A1:D2"/>
-    <mergeCell ref="E1:U1"/>
-    <mergeCell ref="E2:U2"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="R37:U39"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="M10:O10"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="M13:O13"/>
-    <mergeCell ref="P13:R13"/>
-    <mergeCell ref="S13:U13"/>
-    <mergeCell ref="A14:C14"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
feat: change battery download template
</commit_message>
<xml_diff>
--- a/public/assets/templates/maintenance/battery.xlsx
+++ b/public/assets/templates/maintenance/battery.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\maintenance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA4143BF-B41D-411B-A1D3-033153053317}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ED11AA5-EC68-4AE0-B787-9A9C933D7005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{632ED090-5FEF-4C64-87E3-52D42BEDE752}"/>
   </bookViews>
@@ -457,7 +457,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -509,8 +509,68 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -527,15 +587,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -544,60 +595,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -980,54 +977,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="15" thickTop="1">
-      <c r="A1" s="35"/>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="38" t="s">
+      <c r="A1" s="25"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
-      <c r="L1" s="39"/>
-      <c r="M1" s="39"/>
-      <c r="N1" s="39"/>
-      <c r="O1" s="39"/>
-      <c r="P1" s="39"/>
-      <c r="Q1" s="39"/>
-      <c r="R1" s="39"/>
-      <c r="S1" s="39"/>
-      <c r="T1" s="39"/>
-      <c r="U1" s="40"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
+      <c r="O1" s="30"/>
+      <c r="P1" s="30"/>
+      <c r="Q1" s="30"/>
+      <c r="R1" s="30"/>
+      <c r="S1" s="30"/>
+      <c r="T1" s="30"/>
+      <c r="U1" s="31"/>
     </row>
     <row r="2" spans="1:21">
-      <c r="A2" s="37"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="41" t="s">
+      <c r="A2" s="27"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="42"/>
-      <c r="L2" s="42"/>
-      <c r="M2" s="42"/>
-      <c r="N2" s="42"/>
-      <c r="O2" s="42"/>
-      <c r="P2" s="42"/>
-      <c r="Q2" s="42"/>
-      <c r="R2" s="42"/>
-      <c r="S2" s="42"/>
-      <c r="T2" s="42"/>
-      <c r="U2" s="43"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="33"/>
+      <c r="N2" s="33"/>
+      <c r="O2" s="33"/>
+      <c r="P2" s="33"/>
+      <c r="Q2" s="33"/>
+      <c r="R2" s="33"/>
+      <c r="S2" s="33"/>
+      <c r="T2" s="33"/>
+      <c r="U2" s="34"/>
     </row>
     <row r="3" spans="1:21">
       <c r="A3" s="1"/>
@@ -1035,28 +1032,28 @@
       <c r="U3" s="3"/>
     </row>
     <row r="4" spans="1:21">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
       <c r="G4" s="4"/>
       <c r="H4" t="s">
         <v>3</v>
       </c>
-      <c r="K4" s="45"/>
-      <c r="L4" s="45"/>
-      <c r="M4" s="45"/>
-      <c r="N4" s="45"/>
+      <c r="K4" s="37"/>
+      <c r="L4" s="37"/>
+      <c r="M4" s="37"/>
+      <c r="N4" s="37"/>
       <c r="P4" t="s">
         <v>4</v>
       </c>
-      <c r="R4" s="45"/>
-      <c r="S4" s="45"/>
-      <c r="T4" s="45"/>
+      <c r="R4" s="37"/>
+      <c r="S4" s="37"/>
+      <c r="T4" s="37"/>
       <c r="U4" s="3"/>
     </row>
     <row r="5" spans="1:21">
@@ -1070,22 +1067,22 @@
       <c r="U5" s="3"/>
     </row>
     <row r="6" spans="1:21">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="24"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="36"/>
+      <c r="D6" s="36"/>
+      <c r="E6" s="36"/>
+      <c r="F6" s="36"/>
       <c r="G6" s="7"/>
       <c r="H6" t="s">
         <v>6</v>
       </c>
-      <c r="K6" s="46"/>
-      <c r="L6" s="46"/>
-      <c r="M6" s="46"/>
-      <c r="N6" s="46"/>
+      <c r="K6" s="37"/>
+      <c r="L6" s="37"/>
+      <c r="M6" s="37"/>
+      <c r="N6" s="37"/>
       <c r="U6" s="3"/>
     </row>
     <row r="7" spans="1:21">
@@ -1105,11 +1102,11 @@
       <c r="U8" s="3"/>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="31" t="s">
+      <c r="A9" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="32"/>
-      <c r="C9" s="32"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
       <c r="D9" s="9" t="s">
         <v>8</v>
       </c>
@@ -1166,61 +1163,61 @@
       </c>
     </row>
     <row r="10" spans="1:21">
-      <c r="A10" s="29" t="s">
+      <c r="A10" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="30"/>
-      <c r="C10" s="30"/>
-      <c r="D10" s="33"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="33"/>
-      <c r="G10" s="33"/>
-      <c r="H10" s="33"/>
-      <c r="I10" s="33"/>
-      <c r="J10" s="33"/>
-      <c r="K10" s="33"/>
-      <c r="L10" s="33"/>
-      <c r="M10" s="33"/>
-      <c r="N10" s="33"/>
-      <c r="O10" s="33"/>
-      <c r="P10" s="33"/>
-      <c r="Q10" s="33"/>
-      <c r="R10" s="33"/>
-      <c r="S10" s="33"/>
-      <c r="T10" s="33"/>
-      <c r="U10" s="34"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="23"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
+      <c r="M10" s="23"/>
+      <c r="N10" s="23"/>
+      <c r="O10" s="23"/>
+      <c r="P10" s="23"/>
+      <c r="Q10" s="23"/>
+      <c r="R10" s="23"/>
+      <c r="S10" s="23"/>
+      <c r="T10" s="23"/>
+      <c r="U10" s="24"/>
     </row>
     <row r="11" spans="1:21">
-      <c r="A11" s="29" t="s">
+      <c r="A11" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="30"/>
-      <c r="C11" s="30"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
-      <c r="K11" s="17"/>
-      <c r="L11" s="17"/>
-      <c r="M11" s="17"/>
-      <c r="N11" s="17"/>
-      <c r="O11" s="17"/>
-      <c r="P11" s="17"/>
-      <c r="Q11" s="17"/>
-      <c r="R11" s="17"/>
-      <c r="S11" s="17"/>
-      <c r="T11" s="17"/>
-      <c r="U11" s="18"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="28"/>
+      <c r="K11" s="28"/>
+      <c r="L11" s="28"/>
+      <c r="M11" s="28"/>
+      <c r="N11" s="28"/>
+      <c r="O11" s="28"/>
+      <c r="P11" s="28"/>
+      <c r="Q11" s="28"/>
+      <c r="R11" s="28"/>
+      <c r="S11" s="28"/>
+      <c r="T11" s="28"/>
+      <c r="U11" s="38"/>
     </row>
     <row r="12" spans="1:21">
-      <c r="A12" s="31" t="s">
+      <c r="A12" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="32"/>
-      <c r="C12" s="32"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
       <c r="D12" s="12" t="s">
         <v>8</v>
       </c>
@@ -1277,61 +1274,61 @@
       </c>
     </row>
     <row r="13" spans="1:21">
-      <c r="A13" s="29" t="s">
+      <c r="A13" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="30"/>
-      <c r="C13" s="30"/>
-      <c r="D13" s="33"/>
-      <c r="E13" s="33"/>
-      <c r="F13" s="33"/>
-      <c r="G13" s="33"/>
-      <c r="H13" s="33"/>
-      <c r="I13" s="33"/>
-      <c r="J13" s="33"/>
-      <c r="K13" s="33"/>
-      <c r="L13" s="33"/>
-      <c r="M13" s="33"/>
-      <c r="N13" s="33"/>
-      <c r="O13" s="33"/>
-      <c r="P13" s="33"/>
-      <c r="Q13" s="33"/>
-      <c r="R13" s="33"/>
-      <c r="S13" s="33"/>
-      <c r="T13" s="33"/>
-      <c r="U13" s="34"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="23"/>
+      <c r="I13" s="23"/>
+      <c r="J13" s="23"/>
+      <c r="K13" s="23"/>
+      <c r="L13" s="23"/>
+      <c r="M13" s="23"/>
+      <c r="N13" s="23"/>
+      <c r="O13" s="23"/>
+      <c r="P13" s="23"/>
+      <c r="Q13" s="23"/>
+      <c r="R13" s="23"/>
+      <c r="S13" s="23"/>
+      <c r="T13" s="23"/>
+      <c r="U13" s="24"/>
     </row>
     <row r="14" spans="1:21">
-      <c r="A14" s="29" t="s">
+      <c r="A14" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="30"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="17"/>
-      <c r="L14" s="17"/>
-      <c r="M14" s="17"/>
-      <c r="N14" s="17"/>
-      <c r="O14" s="17"/>
-      <c r="P14" s="17"/>
-      <c r="Q14" s="17"/>
-      <c r="R14" s="17"/>
-      <c r="S14" s="17"/>
-      <c r="T14" s="17"/>
-      <c r="U14" s="18"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="28"/>
+      <c r="J14" s="28"/>
+      <c r="K14" s="28"/>
+      <c r="L14" s="28"/>
+      <c r="M14" s="28"/>
+      <c r="N14" s="28"/>
+      <c r="O14" s="28"/>
+      <c r="P14" s="28"/>
+      <c r="Q14" s="28"/>
+      <c r="R14" s="28"/>
+      <c r="S14" s="28"/>
+      <c r="T14" s="28"/>
+      <c r="U14" s="38"/>
     </row>
     <row r="15" spans="1:21">
-      <c r="A15" s="31" t="s">
+      <c r="A15" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="32"/>
-      <c r="C15" s="32"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
       <c r="D15" s="12" t="s">
         <v>8</v>
       </c>
@@ -1388,61 +1385,61 @@
       </c>
     </row>
     <row r="16" spans="1:21">
-      <c r="A16" s="29" t="s">
+      <c r="A16" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="33"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="33"/>
-      <c r="H16" s="33"/>
-      <c r="I16" s="33"/>
-      <c r="J16" s="33"/>
-      <c r="K16" s="33"/>
-      <c r="L16" s="33"/>
-      <c r="M16" s="33"/>
-      <c r="N16" s="33"/>
-      <c r="O16" s="33"/>
-      <c r="P16" s="33"/>
-      <c r="Q16" s="33"/>
-      <c r="R16" s="33"/>
-      <c r="S16" s="33"/>
-      <c r="T16" s="33"/>
-      <c r="U16" s="34"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="23"/>
+      <c r="M16" s="23"/>
+      <c r="N16" s="23"/>
+      <c r="O16" s="23"/>
+      <c r="P16" s="23"/>
+      <c r="Q16" s="23"/>
+      <c r="R16" s="23"/>
+      <c r="S16" s="23"/>
+      <c r="T16" s="23"/>
+      <c r="U16" s="24"/>
     </row>
     <row r="17" spans="1:21">
-      <c r="A17" s="29" t="s">
+      <c r="A17" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="30"/>
-      <c r="C17" s="30"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="17"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="17"/>
-      <c r="K17" s="17"/>
-      <c r="L17" s="17"/>
-      <c r="M17" s="17"/>
-      <c r="N17" s="17"/>
-      <c r="O17" s="17"/>
-      <c r="P17" s="17"/>
-      <c r="Q17" s="17"/>
-      <c r="R17" s="17"/>
-      <c r="S17" s="17"/>
-      <c r="T17" s="17"/>
-      <c r="U17" s="18"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="28"/>
+      <c r="I17" s="28"/>
+      <c r="J17" s="28"/>
+      <c r="K17" s="28"/>
+      <c r="L17" s="28"/>
+      <c r="M17" s="28"/>
+      <c r="N17" s="28"/>
+      <c r="O17" s="28"/>
+      <c r="P17" s="28"/>
+      <c r="Q17" s="28"/>
+      <c r="R17" s="28"/>
+      <c r="S17" s="28"/>
+      <c r="T17" s="28"/>
+      <c r="U17" s="38"/>
     </row>
     <row r="18" spans="1:21">
-      <c r="A18" s="31" t="s">
+      <c r="A18" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="32"/>
-      <c r="C18" s="32"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
       <c r="D18" s="12" t="s">
         <v>8</v>
       </c>
@@ -1499,54 +1496,54 @@
       </c>
     </row>
     <row r="19" spans="1:21">
-      <c r="A19" s="29" t="s">
+      <c r="A19" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B19" s="30"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="33"/>
-      <c r="E19" s="33"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="33"/>
-      <c r="H19" s="33"/>
-      <c r="I19" s="33"/>
-      <c r="J19" s="33"/>
-      <c r="K19" s="33"/>
-      <c r="L19" s="33"/>
-      <c r="M19" s="33"/>
-      <c r="N19" s="33"/>
-      <c r="O19" s="33"/>
-      <c r="P19" s="33"/>
-      <c r="Q19" s="33"/>
-      <c r="R19" s="33"/>
-      <c r="S19" s="33"/>
-      <c r="T19" s="33"/>
-      <c r="U19" s="34"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
+      <c r="G19" s="23"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
+      <c r="J19" s="23"/>
+      <c r="K19" s="23"/>
+      <c r="L19" s="23"/>
+      <c r="M19" s="23"/>
+      <c r="N19" s="23"/>
+      <c r="O19" s="23"/>
+      <c r="P19" s="23"/>
+      <c r="Q19" s="23"/>
+      <c r="R19" s="23"/>
+      <c r="S19" s="23"/>
+      <c r="T19" s="23"/>
+      <c r="U19" s="24"/>
     </row>
     <row r="20" spans="1:21">
-      <c r="A20" s="29" t="s">
+      <c r="A20" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="30"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="17"/>
-      <c r="K20" s="17"/>
-      <c r="L20" s="17"/>
-      <c r="M20" s="17"/>
-      <c r="N20" s="17"/>
-      <c r="O20" s="17"/>
-      <c r="P20" s="17"/>
-      <c r="Q20" s="17"/>
-      <c r="R20" s="17"/>
-      <c r="S20" s="17"/>
-      <c r="T20" s="17"/>
-      <c r="U20" s="18"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
+      <c r="I20" s="28"/>
+      <c r="J20" s="28"/>
+      <c r="K20" s="28"/>
+      <c r="L20" s="28"/>
+      <c r="M20" s="28"/>
+      <c r="N20" s="28"/>
+      <c r="O20" s="28"/>
+      <c r="P20" s="28"/>
+      <c r="Q20" s="28"/>
+      <c r="R20" s="28"/>
+      <c r="S20" s="28"/>
+      <c r="T20" s="28"/>
+      <c r="U20" s="38"/>
     </row>
     <row r="21" spans="1:21">
       <c r="A21" s="1"/>
@@ -1653,98 +1650,98 @@
       <c r="U29" s="3"/>
     </row>
     <row r="30" spans="1:21">
-      <c r="A30" s="20" t="s">
+      <c r="A30" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="B30" s="21"/>
-      <c r="C30" s="21"/>
-      <c r="D30" s="21"/>
-      <c r="E30" s="21"/>
-      <c r="F30" s="21"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="21"/>
-      <c r="I30" s="21"/>
-      <c r="J30" s="21"/>
-      <c r="K30" s="21"/>
-      <c r="L30" s="21"/>
-      <c r="M30" s="21"/>
-      <c r="N30" s="21"/>
-      <c r="O30" s="21"/>
-      <c r="P30" s="21"/>
-      <c r="Q30" s="21"/>
-      <c r="R30" s="21"/>
-      <c r="S30" s="21"/>
-      <c r="T30" s="21"/>
-      <c r="U30" s="22"/>
+      <c r="B30" s="41"/>
+      <c r="C30" s="41"/>
+      <c r="D30" s="41"/>
+      <c r="E30" s="41"/>
+      <c r="F30" s="41"/>
+      <c r="G30" s="41"/>
+      <c r="H30" s="41"/>
+      <c r="I30" s="41"/>
+      <c r="J30" s="41"/>
+      <c r="K30" s="41"/>
+      <c r="L30" s="41"/>
+      <c r="M30" s="41"/>
+      <c r="N30" s="41"/>
+      <c r="O30" s="41"/>
+      <c r="P30" s="41"/>
+      <c r="Q30" s="41"/>
+      <c r="R30" s="41"/>
+      <c r="S30" s="41"/>
+      <c r="T30" s="41"/>
+      <c r="U30" s="42"/>
     </row>
     <row r="31" spans="1:21">
-      <c r="A31" s="20"/>
-      <c r="B31" s="21"/>
-      <c r="C31" s="21"/>
-      <c r="D31" s="21"/>
-      <c r="E31" s="21"/>
-      <c r="F31" s="21"/>
-      <c r="G31" s="21"/>
-      <c r="H31" s="21"/>
-      <c r="I31" s="21"/>
-      <c r="J31" s="21"/>
-      <c r="K31" s="21"/>
-      <c r="L31" s="21"/>
-      <c r="M31" s="21"/>
-      <c r="N31" s="21"/>
-      <c r="O31" s="21"/>
-      <c r="P31" s="21"/>
-      <c r="Q31" s="21"/>
-      <c r="R31" s="21"/>
-      <c r="S31" s="21"/>
-      <c r="T31" s="21"/>
-      <c r="U31" s="22"/>
+      <c r="A31" s="40"/>
+      <c r="B31" s="41"/>
+      <c r="C31" s="41"/>
+      <c r="D31" s="41"/>
+      <c r="E31" s="41"/>
+      <c r="F31" s="41"/>
+      <c r="G31" s="41"/>
+      <c r="H31" s="41"/>
+      <c r="I31" s="41"/>
+      <c r="J31" s="41"/>
+      <c r="K31" s="41"/>
+      <c r="L31" s="41"/>
+      <c r="M31" s="41"/>
+      <c r="N31" s="41"/>
+      <c r="O31" s="41"/>
+      <c r="P31" s="41"/>
+      <c r="Q31" s="41"/>
+      <c r="R31" s="41"/>
+      <c r="S31" s="41"/>
+      <c r="T31" s="41"/>
+      <c r="U31" s="42"/>
     </row>
     <row r="32" spans="1:21">
-      <c r="A32" s="20"/>
-      <c r="B32" s="21"/>
-      <c r="C32" s="21"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
-      <c r="H32" s="21"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="21"/>
-      <c r="K32" s="21"/>
-      <c r="L32" s="21"/>
-      <c r="M32" s="21"/>
-      <c r="N32" s="21"/>
-      <c r="O32" s="21"/>
-      <c r="P32" s="21"/>
-      <c r="Q32" s="21"/>
-      <c r="R32" s="21"/>
-      <c r="S32" s="21"/>
-      <c r="T32" s="21"/>
-      <c r="U32" s="22"/>
+      <c r="A32" s="40"/>
+      <c r="B32" s="41"/>
+      <c r="C32" s="41"/>
+      <c r="D32" s="41"/>
+      <c r="E32" s="41"/>
+      <c r="F32" s="41"/>
+      <c r="G32" s="41"/>
+      <c r="H32" s="41"/>
+      <c r="I32" s="41"/>
+      <c r="J32" s="41"/>
+      <c r="K32" s="41"/>
+      <c r="L32" s="41"/>
+      <c r="M32" s="41"/>
+      <c r="N32" s="41"/>
+      <c r="O32" s="41"/>
+      <c r="P32" s="41"/>
+      <c r="Q32" s="41"/>
+      <c r="R32" s="41"/>
+      <c r="S32" s="41"/>
+      <c r="T32" s="41"/>
+      <c r="U32" s="42"/>
     </row>
     <row r="33" spans="1:21">
-      <c r="A33" s="20"/>
-      <c r="B33" s="21"/>
-      <c r="C33" s="21"/>
-      <c r="D33" s="21"/>
-      <c r="E33" s="21"/>
-      <c r="F33" s="21"/>
-      <c r="G33" s="21"/>
-      <c r="H33" s="21"/>
-      <c r="I33" s="21"/>
-      <c r="J33" s="21"/>
-      <c r="K33" s="21"/>
-      <c r="L33" s="21"/>
-      <c r="M33" s="21"/>
-      <c r="N33" s="21"/>
-      <c r="O33" s="21"/>
-      <c r="P33" s="21"/>
-      <c r="Q33" s="21"/>
-      <c r="R33" s="21"/>
-      <c r="S33" s="21"/>
-      <c r="T33" s="21"/>
-      <c r="U33" s="22"/>
+      <c r="A33" s="40"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="41"/>
+      <c r="H33" s="41"/>
+      <c r="I33" s="41"/>
+      <c r="J33" s="41"/>
+      <c r="K33" s="41"/>
+      <c r="L33" s="41"/>
+      <c r="M33" s="41"/>
+      <c r="N33" s="41"/>
+      <c r="O33" s="41"/>
+      <c r="P33" s="41"/>
+      <c r="Q33" s="41"/>
+      <c r="R33" s="41"/>
+      <c r="S33" s="41"/>
+      <c r="T33" s="41"/>
+      <c r="U33" s="42"/>
     </row>
     <row r="34" spans="1:21">
       <c r="A34" s="1"/>
@@ -1755,107 +1752,172 @@
       <c r="U35" s="3"/>
     </row>
     <row r="36" spans="1:21">
-      <c r="A36" s="23" t="s">
+      <c r="A36" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="B36" s="24"/>
-      <c r="C36" s="24"/>
-      <c r="D36" s="24"/>
-      <c r="J36" s="24" t="s">
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="J36" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K36" s="24"/>
-      <c r="L36" s="24"/>
-      <c r="M36" s="24"/>
-      <c r="R36" s="24" t="s">
+      <c r="K36" s="17"/>
+      <c r="L36" s="17"/>
+      <c r="M36" s="17"/>
+      <c r="R36" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="S36" s="24"/>
-      <c r="T36" s="24"/>
-      <c r="U36" s="25"/>
+      <c r="S36" s="17"/>
+      <c r="T36" s="17"/>
+      <c r="U36" s="18"/>
     </row>
     <row r="37" spans="1:21">
-      <c r="A37" s="23"/>
-      <c r="B37" s="24"/>
-      <c r="C37" s="24"/>
-      <c r="D37" s="24"/>
-      <c r="J37" s="24"/>
-      <c r="K37" s="24"/>
-      <c r="L37" s="24"/>
-      <c r="M37" s="24"/>
-      <c r="R37" s="24"/>
-      <c r="S37" s="24"/>
-      <c r="T37" s="24"/>
-      <c r="U37" s="25"/>
+      <c r="A37" s="35"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="J37" s="17"/>
+      <c r="K37" s="17"/>
+      <c r="L37" s="17"/>
+      <c r="M37" s="17"/>
+      <c r="R37" s="17"/>
+      <c r="S37" s="17"/>
+      <c r="T37" s="17"/>
+      <c r="U37" s="18"/>
     </row>
     <row r="38" spans="1:21">
-      <c r="A38" s="23"/>
-      <c r="B38" s="24"/>
-      <c r="C38" s="24"/>
-      <c r="D38" s="24"/>
-      <c r="J38" s="24"/>
-      <c r="K38" s="24"/>
-      <c r="L38" s="24"/>
-      <c r="M38" s="24"/>
-      <c r="R38" s="24"/>
-      <c r="S38" s="24"/>
-      <c r="T38" s="24"/>
-      <c r="U38" s="25"/>
+      <c r="A38" s="35"/>
+      <c r="B38" s="17"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="J38" s="17"/>
+      <c r="K38" s="17"/>
+      <c r="L38" s="17"/>
+      <c r="M38" s="17"/>
+      <c r="R38" s="17"/>
+      <c r="S38" s="17"/>
+      <c r="T38" s="17"/>
+      <c r="U38" s="18"/>
     </row>
     <row r="39" spans="1:21">
-      <c r="A39" s="23"/>
-      <c r="B39" s="24"/>
-      <c r="C39" s="24"/>
-      <c r="D39" s="24"/>
-      <c r="J39" s="24"/>
-      <c r="K39" s="24"/>
-      <c r="L39" s="24"/>
-      <c r="M39" s="24"/>
-      <c r="R39" s="24"/>
-      <c r="S39" s="24"/>
-      <c r="T39" s="24"/>
-      <c r="U39" s="25"/>
+      <c r="A39" s="35"/>
+      <c r="B39" s="17"/>
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="J39" s="17"/>
+      <c r="K39" s="17"/>
+      <c r="L39" s="17"/>
+      <c r="M39" s="17"/>
+      <c r="R39" s="17"/>
+      <c r="S39" s="17"/>
+      <c r="T39" s="17"/>
+      <c r="U39" s="18"/>
     </row>
     <row r="40" spans="1:21" ht="15" thickBot="1">
-      <c r="A40" s="26" t="s">
+      <c r="A40" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="B40" s="27"/>
-      <c r="C40" s="27"/>
-      <c r="D40" s="27"/>
+      <c r="B40" s="44"/>
+      <c r="C40" s="44"/>
+      <c r="D40" s="44"/>
       <c r="E40" s="15"/>
       <c r="F40" s="15"/>
       <c r="G40" s="15"/>
       <c r="H40" s="15"/>
       <c r="I40" s="15"/>
-      <c r="J40" s="27" t="s">
+      <c r="J40" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="K40" s="27"/>
-      <c r="L40" s="27"/>
-      <c r="M40" s="27"/>
+      <c r="K40" s="44"/>
+      <c r="L40" s="44"/>
+      <c r="M40" s="44"/>
       <c r="N40" s="15"/>
       <c r="O40" s="15"/>
       <c r="P40" s="15"/>
       <c r="Q40" s="15"/>
-      <c r="R40" s="27" t="s">
+      <c r="R40" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="S40" s="27"/>
-      <c r="T40" s="27"/>
-      <c r="U40" s="28"/>
+      <c r="S40" s="44"/>
+      <c r="T40" s="44"/>
+      <c r="U40" s="45"/>
     </row>
     <row r="41" spans="1:21" ht="15" thickTop="1">
-      <c r="Q41" s="19" t="s">
+      <c r="Q41" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="R41" s="19"/>
-      <c r="S41" s="19"/>
-      <c r="T41" s="19"/>
-      <c r="U41" s="19"/>
+      <c r="R41" s="39"/>
+      <c r="S41" s="39"/>
+      <c r="T41" s="39"/>
+      <c r="U41" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="81">
+    <mergeCell ref="P20:R20"/>
+    <mergeCell ref="S20:U20"/>
+    <mergeCell ref="Q41:U41"/>
+    <mergeCell ref="A30:U33"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="J36:M36"/>
+    <mergeCell ref="R36:U36"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="J40:M40"/>
+    <mergeCell ref="R40:U40"/>
+    <mergeCell ref="J37:M39"/>
+    <mergeCell ref="A37:D39"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="M20:O20"/>
+    <mergeCell ref="P17:R17"/>
+    <mergeCell ref="S17:U17"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="P19:R19"/>
+    <mergeCell ref="S19:U19"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="M17:O17"/>
+    <mergeCell ref="S14:U14"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="J16:L16"/>
+    <mergeCell ref="M16:O16"/>
+    <mergeCell ref="P16:R16"/>
+    <mergeCell ref="S16:U16"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="M14:O14"/>
+    <mergeCell ref="P14:R14"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="P10:R10"/>
+    <mergeCell ref="S10:U10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="P11:R11"/>
+    <mergeCell ref="S11:U11"/>
+    <mergeCell ref="K6:N6"/>
+    <mergeCell ref="A1:D2"/>
+    <mergeCell ref="E1:U1"/>
+    <mergeCell ref="E2:U2"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="K4:N4"/>
+    <mergeCell ref="R4:T4"/>
     <mergeCell ref="R37:U39"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A10:C10"/>
@@ -1872,71 +1934,6 @@
     <mergeCell ref="P13:R13"/>
     <mergeCell ref="S13:U13"/>
     <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A1:D2"/>
-    <mergeCell ref="E1:U1"/>
-    <mergeCell ref="E2:U2"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="K4:N4"/>
-    <mergeCell ref="R4:T4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="P10:R10"/>
-    <mergeCell ref="S10:U10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="P11:R11"/>
-    <mergeCell ref="S11:U11"/>
-    <mergeCell ref="K6:N6"/>
-    <mergeCell ref="S14:U14"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="J16:L16"/>
-    <mergeCell ref="M16:O16"/>
-    <mergeCell ref="P16:R16"/>
-    <mergeCell ref="S16:U16"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="M14:O14"/>
-    <mergeCell ref="P14:R14"/>
-    <mergeCell ref="M20:O20"/>
-    <mergeCell ref="P17:R17"/>
-    <mergeCell ref="S17:U17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="P19:R19"/>
-    <mergeCell ref="S19:U19"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="M17:O17"/>
-    <mergeCell ref="P20:R20"/>
-    <mergeCell ref="S20:U20"/>
-    <mergeCell ref="Q41:U41"/>
-    <mergeCell ref="A30:U33"/>
-    <mergeCell ref="A36:D36"/>
-    <mergeCell ref="J36:M36"/>
-    <mergeCell ref="R36:U36"/>
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="J40:M40"/>
-    <mergeCell ref="R40:U40"/>
-    <mergeCell ref="J37:M39"/>
-    <mergeCell ref="A37:D39"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="J20:L20"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>